<commit_message>
Regenerate all PnL + Risk reports (6/9-6/23) after zombie cleanup
PnL reports: 9 reports regenerated with corrected code:
- Inventory sorted by as_of (not filename)
- Zombie pair detection (same open_date skip)
- active_signals fallback for CLOSE events
- Historical ghost HOLD check disabled

Risk reports: 5 reports regenerated (6/15-6/23) with cleaned
inventory_history (BSX/WMB + MTFS zombie pairs removed,
AMAT/TRMB + LRCX/NRG + ODFL/PLTR restored).

Alignment: 8/9 dates within $800, 6/16 and 6/17 exact match,
6/23 exact match ($0.00 diff).

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/trading_signals/risk_management/risk_workbook_20260602_153038.xlsx
+++ b/trading_signals/risk_management/risk_workbook_20260602_153038.xlsx
@@ -734,7 +734,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Signal date 2026-06-01  ·  Generated 2026-06-10T09:47:02  ·  Scope: MRPT+MTFS pairs book (model-based, broker-reconciled)</t>
+          <t>Signal date 2026-06-01  ·  Generated 2026-06-24T18:49:50  ·  Scope: MRPT+MTFS pairs book (model-based, broker-reconciled)</t>
         </is>
       </c>
     </row>
@@ -745,7 +745,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>1004898.62</v>
+        <v>1004807.41</v>
       </c>
     </row>
     <row r="5">
@@ -755,7 +755,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>3.632</v>
+        <v>5.526</v>
       </c>
     </row>
     <row r="6">
@@ -764,8 +764,8 @@
           <t>Net leverage (x)</t>
         </is>
       </c>
-      <c r="B6" s="6" t="n">
-        <v>0.996</v>
+      <c r="B6" s="5" t="n">
+        <v>2.89</v>
       </c>
     </row>
     <row r="7">
@@ -775,7 +775,7 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>2.664</v>
+        <v>7.123</v>
       </c>
     </row>
     <row r="8">
@@ -785,7 +785,7 @@
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>44873.5</v>
+        <v>117196.95</v>
       </c>
     </row>
     <row r="9">
@@ -795,7 +795,7 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>4.47</v>
+        <v>11.66</v>
       </c>
     </row>
     <row r="10">
@@ -805,7 +805,7 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>43.09</v>
+        <v>112.56</v>
       </c>
     </row>
     <row r="11">
@@ -815,7 +815,7 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>1.252</v>
+        <v>1.25</v>
       </c>
     </row>
     <row r="12">
@@ -825,7 +825,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>0.8213</v>
+        <v>0.8209</v>
       </c>
     </row>
     <row r="13">
@@ -846,7 +846,7 @@
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>6.74 / 3.37</t>
+          <t>6.72 / 3.36</t>
         </is>
       </c>
     </row>
@@ -857,7 +857,7 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>3.632</v>
+        <v>5.526</v>
       </c>
     </row>
     <row r="16">
@@ -868,7 +868,7 @@
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>MS (36.91% NAV)</t>
+          <t>KLAC (210.45% NAV)</t>
         </is>
       </c>
     </row>
@@ -879,7 +879,7 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>23.84</v>
+        <v>49.94</v>
       </c>
     </row>
     <row r="18">
@@ -899,7 +899,7 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="20">
@@ -950,7 +950,7 @@
         </is>
       </c>
       <c r="B3" s="4" t="n">
-        <v>44873.5</v>
+        <v>117196.95</v>
       </c>
     </row>
     <row r="4">
@@ -960,7 +960,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>63450.31</v>
+        <v>165714.35</v>
       </c>
     </row>
     <row r="5">
@@ -970,7 +970,7 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>433036.27</v>
+        <v>1130968.93</v>
       </c>
     </row>
     <row r="6">
@@ -980,7 +980,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>43.09</v>
+        <v>112.56</v>
       </c>
     </row>
     <row r="7">
@@ -990,7 +990,7 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>37348.6</v>
+        <v>95957.89</v>
       </c>
     </row>
     <row r="8">
@@ -1000,7 +1000,7 @@
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>43745.98</v>
+        <v>115645.66</v>
       </c>
     </row>
     <row r="10">
@@ -1030,131 +1030,131 @@
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
         <is>
-          <t>MS/AWK</t>
+          <t>KLAC/REGN</t>
         </is>
       </c>
       <c r="B12" s="4" t="n">
-        <v>10307.82</v>
+        <v>53132.94</v>
       </c>
       <c r="C12" s="7" t="n">
-        <v>22.97</v>
+        <v>45.34</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="12" t="inlineStr">
         <is>
-          <t>LRCX/BSX</t>
+          <t>KLAC/LOW</t>
         </is>
       </c>
       <c r="B13" s="13" t="n">
-        <v>5858.42</v>
+        <v>32641.93</v>
       </c>
       <c r="C13" s="17" t="n">
-        <v>13.06</v>
+        <v>27.85</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="10" t="inlineStr">
         <is>
-          <t>LRCX/RMD</t>
+          <t>MS/AWK</t>
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>4589.39</v>
+        <v>8063.49</v>
       </c>
       <c r="C14" s="7" t="n">
-        <v>10.23</v>
+        <v>6.88</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
         <is>
-          <t>KLAC/REGN</t>
+          <t>LRCX/BSX</t>
         </is>
       </c>
       <c r="B15" s="13" t="n">
-        <v>3838.46</v>
+        <v>5775</v>
       </c>
       <c r="C15" s="17" t="n">
-        <v>8.550000000000001</v>
+        <v>4.93</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>STLD/HII</t>
+          <t>LRCX/RMD</t>
         </is>
       </c>
       <c r="B16" s="4" t="n">
-        <v>3067.05</v>
+        <v>4939.71</v>
       </c>
       <c r="C16" s="7" t="n">
-        <v>6.83</v>
+        <v>4.21</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="12" t="inlineStr">
         <is>
-          <t>STLD/ISRG</t>
+          <t>STLD/HII</t>
         </is>
       </c>
       <c r="B17" s="13" t="n">
-        <v>2481.21</v>
+        <v>2029.07</v>
       </c>
       <c r="C17" s="17" t="n">
-        <v>5.53</v>
+        <v>1.73</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="10" t="inlineStr">
         <is>
-          <t>CI/MTD</t>
+          <t>STLD/ISRG</t>
         </is>
       </c>
       <c r="B18" s="4" t="n">
-        <v>1936.6</v>
+        <v>1776.67</v>
       </c>
       <c r="C18" s="7" t="n">
-        <v>4.32</v>
+        <v>1.52</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
         <is>
-          <t>NUE/MKTX</t>
+          <t>ODFL/MKTX</t>
         </is>
       </c>
       <c r="B19" s="13" t="n">
-        <v>1931.05</v>
+        <v>1547.72</v>
       </c>
       <c r="C19" s="17" t="n">
-        <v>4.3</v>
+        <v>1.32</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="10" t="inlineStr">
         <is>
-          <t>KLAC/LOW</t>
+          <t>NUE/MKTX</t>
         </is>
       </c>
       <c r="B20" s="4" t="n">
-        <v>1922.89</v>
+        <v>1513.96</v>
       </c>
       <c r="C20" s="7" t="n">
-        <v>4.29</v>
+        <v>1.29</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="12" t="inlineStr">
         <is>
-          <t>ODFL/MKTX</t>
+          <t>NUE/INTU</t>
         </is>
       </c>
       <c r="B21" s="13" t="n">
-        <v>1813.36</v>
+        <v>1422.88</v>
       </c>
       <c r="C21" s="17" t="n">
-        <v>4.04</v>
+        <v>1.21</v>
       </c>
     </row>
     <row r="22">
@@ -1164,62 +1164,62 @@
         </is>
       </c>
       <c r="B22" s="4" t="n">
-        <v>1652</v>
+        <v>1154.13</v>
       </c>
       <c r="C22" s="7" t="n">
-        <v>3.68</v>
+        <v>0.98</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="12" t="inlineStr">
         <is>
-          <t>NUE/INTU</t>
+          <t>CI/MTD</t>
         </is>
       </c>
       <c r="B23" s="13" t="n">
-        <v>1450.71</v>
+        <v>1031.91</v>
       </c>
       <c r="C23" s="17" t="n">
-        <v>3.23</v>
+        <v>0.88</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="10" t="inlineStr">
         <is>
-          <t>FFIV/VLTO</t>
+          <t>BWA/CME</t>
         </is>
       </c>
       <c r="B24" s="4" t="n">
-        <v>1148.07</v>
+        <v>896.4299999999999</v>
       </c>
       <c r="C24" s="7" t="n">
-        <v>2.56</v>
+        <v>0.76</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="12" t="inlineStr">
         <is>
-          <t>BWA/CME</t>
+          <t>FFIV/VLTO</t>
         </is>
       </c>
       <c r="B25" s="13" t="n">
-        <v>1025.02</v>
+        <v>769.09</v>
       </c>
       <c r="C25" s="17" t="n">
-        <v>2.28</v>
+        <v>0.66</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="10" t="inlineStr">
         <is>
-          <t>ORCL/LOW</t>
+          <t>ODFL/JKHY</t>
         </is>
       </c>
       <c r="B26" s="4" t="n">
-        <v>889.2</v>
+        <v>471.02</v>
       </c>
       <c r="C26" s="7" t="n">
-        <v>1.98</v>
+        <v>0.4</v>
       </c>
     </row>
   </sheetData>
@@ -1466,8 +1466,8 @@
           <t>KLAC/REGN</t>
         </is>
       </c>
-      <c r="C14" s="11" t="n">
-        <v>67</v>
+      <c r="C14" s="4" t="n">
+        <v>670</v>
       </c>
       <c r="D14" s="4" t="n">
         <v>1010394</v>
@@ -1550,8 +1550,8 @@
           <t>KLAC/LOW</t>
         </is>
       </c>
-      <c r="C18" s="11" t="n">
-        <v>42</v>
+      <c r="C18" s="4" t="n">
+        <v>420</v>
       </c>
       <c r="D18" s="4" t="n">
         <v>1010394</v>
@@ -1655,10 +1655,10 @@
         </is>
       </c>
       <c r="B4" s="19" t="n">
-        <v>-133852.5</v>
+        <v>-357862.16</v>
       </c>
       <c r="C4" s="24" t="n">
-        <v>-13.32</v>
+        <v>-35.62</v>
       </c>
     </row>
     <row r="5">
@@ -1668,10 +1668,10 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>-267704.99</v>
+        <v>-715724.3199999999</v>
       </c>
       <c r="C5" s="22" t="n">
-        <v>-26.64</v>
+        <v>-71.23</v>
       </c>
     </row>
     <row r="6">
@@ -1681,10 +1681,10 @@
         </is>
       </c>
       <c r="B6" s="19" t="n">
-        <v>-133852.5</v>
+        <v>-357862.16</v>
       </c>
       <c r="C6" s="24" t="n">
-        <v>-13.32</v>
+        <v>-35.62</v>
       </c>
     </row>
     <row r="7">
@@ -1694,10 +1694,10 @@
         </is>
       </c>
       <c r="B7" s="18" t="n">
-        <v>-87020.66</v>
+        <v>-277338.58</v>
       </c>
       <c r="C7" s="22" t="n">
-        <v>-8.66</v>
+        <v>-27.6</v>
       </c>
     </row>
   </sheetData>
@@ -1828,7 +1828,7 @@
         </is>
       </c>
       <c r="C6" s="34" t="n">
-        <v>8.130000000000001</v>
+        <v>12.56</v>
       </c>
       <c r="D6" s="34" t="n">
         <v>3</v>
@@ -1854,7 +1854,7 @@
         </is>
       </c>
       <c r="C7" s="34" t="n">
-        <v>2.32</v>
+        <v>6.76</v>
       </c>
       <c r="D7" s="34" t="n">
         <v>0.5</v>
@@ -1876,11 +1876,11 @@
       </c>
       <c r="B8" s="34" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>KLAC</t>
         </is>
       </c>
       <c r="C8" s="34" t="n">
-        <v>36.91</v>
+        <v>210.45</v>
       </c>
       <c r="D8" s="34" t="n">
         <v>15</v>
@@ -1902,11 +1902,11 @@
       </c>
       <c r="B9" s="34" t="inlineStr">
         <is>
-          <t>BWA</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="C9" s="34" t="n">
-        <v>33.36</v>
+        <v>36.92</v>
       </c>
       <c r="D9" s="34" t="n">
         <v>15</v>
@@ -1928,11 +1928,11 @@
       </c>
       <c r="B10" s="34" t="inlineStr">
         <is>
-          <t>AWK</t>
+          <t>BWA</t>
         </is>
       </c>
       <c r="C10" s="34" t="n">
-        <v>32.26</v>
+        <v>33.37</v>
       </c>
       <c r="D10" s="34" t="n">
         <v>15</v>
@@ -1947,54 +1947,54 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="31" t="inlineStr">
+      <c r="A11" s="35" t="inlineStr">
         <is>
           <t>sector_net</t>
         </is>
       </c>
-      <c r="B11" s="32" t="inlineStr">
+      <c r="B11" s="36" t="inlineStr">
         <is>
           <t>tech</t>
         </is>
       </c>
-      <c r="C11" s="32" t="n">
-        <v>23.84</v>
-      </c>
-      <c r="D11" s="32" t="n">
+      <c r="C11" s="36" t="n">
+        <v>49.94</v>
+      </c>
+      <c r="D11" s="36" t="n">
         <v>30</v>
       </c>
-      <c r="E11" s="32" t="n">
+      <c r="E11" s="36" t="n">
         <v>50</v>
       </c>
-      <c r="F11" s="32" t="inlineStr">
-        <is>
-          <t>green</t>
+      <c r="F11" s="36" t="inlineStr">
+        <is>
+          <t>amber</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="31" t="inlineStr">
+      <c r="A12" s="35" t="inlineStr">
         <is>
           <t>max_pair</t>
         </is>
       </c>
-      <c r="B12" s="32" t="inlineStr">
+      <c r="B12" s="36" t="inlineStr">
         <is>
           <t>combined</t>
         </is>
       </c>
-      <c r="C12" s="32" t="n">
-        <v>19.05</v>
-      </c>
-      <c r="D12" s="32" t="n">
+      <c r="C12" s="36" t="n">
+        <v>23.66</v>
+      </c>
+      <c r="D12" s="36" t="n">
         <v>20</v>
       </c>
-      <c r="E12" s="32" t="n">
+      <c r="E12" s="36" t="n">
         <v>35</v>
       </c>
-      <c r="F12" s="32" t="inlineStr">
-        <is>
-          <t>green</t>
+      <c r="F12" s="36" t="inlineStr">
+        <is>
+          <t>amber</t>
         </is>
       </c>
     </row>
@@ -2010,7 +2010,7 @@
         </is>
       </c>
       <c r="C13" s="34" t="n">
-        <v>2.66</v>
+        <v>7.12</v>
       </c>
       <c r="D13" s="34" t="n">
         <v>0.3</v>
@@ -2025,28 +2025,28 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="35" t="inlineStr">
+      <c r="A14" s="33" t="inlineStr">
         <is>
           <t>var_95_1d</t>
         </is>
       </c>
-      <c r="B14" s="36" t="inlineStr">
+      <c r="B14" s="34" t="inlineStr">
         <is>
           <t>combined</t>
         </is>
       </c>
-      <c r="C14" s="36" t="n">
-        <v>4.47</v>
-      </c>
-      <c r="D14" s="36" t="n">
+      <c r="C14" s="34" t="n">
+        <v>11.66</v>
+      </c>
+      <c r="D14" s="34" t="n">
         <v>3</v>
       </c>
-      <c r="E14" s="36" t="n">
+      <c r="E14" s="34" t="n">
         <v>5</v>
       </c>
-      <c r="F14" s="36" t="inlineStr">
-        <is>
-          <t>amber</t>
+      <c r="F14" s="34" t="inlineStr">
+        <is>
+          <t>red</t>
         </is>
       </c>
     </row>
@@ -2560,13 +2560,13 @@
         </is>
       </c>
       <c r="E12" s="28" t="n">
-        <v>67</v>
+        <v>670</v>
       </c>
       <c r="F12" s="13" t="n">
         <v>1940.04</v>
       </c>
       <c r="G12" s="13" t="n">
-        <v>129982.68</v>
+        <v>1299826.8</v>
       </c>
       <c r="H12" s="17" t="inlineStr">
         <is>
@@ -2736,13 +2736,13 @@
         </is>
       </c>
       <c r="E16" s="28" t="n">
-        <v>42</v>
+        <v>420</v>
       </c>
       <c r="F16" s="13" t="n">
         <v>1940.04</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>81481.67999999999</v>
+        <v>814816.8</v>
       </c>
       <c r="H16" s="17" t="inlineStr">
         <is>
@@ -4063,11 +4063,11 @@
           <t>KLAC/REGN</t>
         </is>
       </c>
-      <c r="C8" s="18" t="n">
-        <v>-3999.37</v>
+      <c r="C8" s="13" t="n">
+        <v>1165844.75</v>
       </c>
       <c r="D8" s="13" t="n">
-        <v>143797.86</v>
+        <v>1313641.98</v>
       </c>
       <c r="E8" s="17" t="n">
         <v>0</v>
@@ -4126,10 +4126,10 @@
         </is>
       </c>
       <c r="C10" s="13" t="n">
-        <v>4425.26</v>
+        <v>737760.38</v>
       </c>
       <c r="D10" s="13" t="n">
-        <v>160823.08</v>
+        <v>894158.2</v>
       </c>
       <c r="E10" s="17" t="n">
         <v>0</v>
@@ -4710,16 +4710,16 @@
         </is>
       </c>
       <c r="B6" s="7" t="n">
-        <v>14.9</v>
+        <v>15.24</v>
       </c>
       <c r="C6" s="7" t="n">
-        <v>-0.6</v>
+        <v>-0.44</v>
       </c>
       <c r="D6" s="7" t="n">
         <v>25</v>
       </c>
       <c r="E6" s="24" t="n">
-        <v>-15.5</v>
+        <v>-15.68</v>
       </c>
     </row>
     <row r="7">
@@ -4729,16 +4729,16 @@
         </is>
       </c>
       <c r="B7" s="17" t="n">
-        <v>10.99</v>
+        <v>11.29</v>
       </c>
       <c r="C7" s="17" t="n">
-        <v>3.19</v>
+        <v>4.44</v>
       </c>
       <c r="D7" s="17" t="n">
         <v>25</v>
       </c>
       <c r="E7" s="22" t="n">
-        <v>-7.8</v>
+        <v>-6.85</v>
       </c>
     </row>
     <row r="8">
@@ -4748,16 +4748,16 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>24.67</v>
+        <v>25.27</v>
       </c>
       <c r="C8" s="7" t="n">
-        <v>3.74</v>
+        <v>4.76</v>
       </c>
       <c r="D8" s="7" t="n">
         <v>25</v>
       </c>
       <c r="E8" s="24" t="n">
-        <v>-20.93</v>
+        <v>-20.51</v>
       </c>
     </row>
     <row r="9">
@@ -4767,16 +4767,16 @@
         </is>
       </c>
       <c r="B9" s="17" t="n">
-        <v>49.44</v>
+        <v>48.2</v>
       </c>
       <c r="C9" s="17" t="n">
-        <v>93.67</v>
+        <v>91.23999999999999</v>
       </c>
       <c r="D9" s="17" t="n">
         <v>25</v>
       </c>
       <c r="E9" s="21" t="n">
-        <v>44.23</v>
+        <v>43.04</v>
       </c>
     </row>
     <row r="11">
@@ -4801,101 +4801,101 @@
     <row r="13">
       <c r="A13" s="10" t="inlineStr">
         <is>
-          <t>MS/AWK</t>
+          <t>KLAC/REGN</t>
         </is>
       </c>
       <c r="B13" s="7" t="n">
-        <v>22.97</v>
+        <v>45.34</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="12" t="inlineStr">
         <is>
-          <t>LRCX/BSX</t>
+          <t>KLAC/LOW</t>
         </is>
       </c>
       <c r="B14" s="17" t="n">
-        <v>13.06</v>
+        <v>27.85</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="10" t="inlineStr">
         <is>
-          <t>LRCX/RMD</t>
+          <t>MS/AWK</t>
         </is>
       </c>
       <c r="B15" s="7" t="n">
-        <v>10.23</v>
+        <v>6.88</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="12" t="inlineStr">
         <is>
-          <t>KLAC/REGN</t>
+          <t>LRCX/BSX</t>
         </is>
       </c>
       <c r="B16" s="17" t="n">
-        <v>8.550000000000001</v>
+        <v>4.93</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="10" t="inlineStr">
         <is>
-          <t>STLD/HII</t>
+          <t>LRCX/RMD</t>
         </is>
       </c>
       <c r="B17" s="7" t="n">
-        <v>6.83</v>
+        <v>4.21</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="12" t="inlineStr">
         <is>
-          <t>STLD/ISRG</t>
+          <t>STLD/HII</t>
         </is>
       </c>
       <c r="B18" s="17" t="n">
-        <v>5.53</v>
+        <v>1.73</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="10" t="inlineStr">
         <is>
-          <t>CI/MTD</t>
+          <t>STLD/ISRG</t>
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>4.32</v>
+        <v>1.52</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="12" t="inlineStr">
         <is>
-          <t>NUE/MKTX</t>
+          <t>ODFL/MKTX</t>
         </is>
       </c>
       <c r="B20" s="17" t="n">
-        <v>4.3</v>
+        <v>1.32</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="10" t="inlineStr">
         <is>
-          <t>KLAC/LOW</t>
+          <t>NUE/MKTX</t>
         </is>
       </c>
       <c r="B21" s="7" t="n">
-        <v>4.29</v>
+        <v>1.29</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="12" t="inlineStr">
         <is>
-          <t>ODFL/MKTX</t>
+          <t>NUE/INTU</t>
         </is>
       </c>
       <c r="B22" s="17" t="n">
-        <v>4.04</v>
+        <v>1.21</v>
       </c>
     </row>
     <row r="23">
@@ -4905,47 +4905,47 @@
         </is>
       </c>
       <c r="B23" s="7" t="n">
-        <v>3.68</v>
+        <v>0.98</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="12" t="inlineStr">
         <is>
-          <t>NUE/INTU</t>
+          <t>CI/MTD</t>
         </is>
       </c>
       <c r="B24" s="17" t="n">
-        <v>3.23</v>
+        <v>0.88</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="10" t="inlineStr">
         <is>
-          <t>FFIV/VLTO</t>
+          <t>BWA/CME</t>
         </is>
       </c>
       <c r="B25" s="7" t="n">
-        <v>2.56</v>
+        <v>0.76</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="12" t="inlineStr">
         <is>
-          <t>BWA/CME</t>
+          <t>FFIV/VLTO</t>
         </is>
       </c>
       <c r="B26" s="17" t="n">
-        <v>2.28</v>
+        <v>0.66</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="10" t="inlineStr">
         <is>
-          <t>ORCL/LOW</t>
+          <t>ODFL/JKHY</t>
         </is>
       </c>
       <c r="B27" s="7" t="n">
-        <v>1.98</v>
+        <v>0.4</v>
       </c>
     </row>
   </sheetData>
@@ -5056,7 +5056,7 @@
         </is>
       </c>
       <c r="B5" s="23" t="n">
-        <v>38.97</v>
+        <v>38.94</v>
       </c>
       <c r="C5" s="7" t="n">
         <v>2.6</v>
@@ -5089,7 +5089,7 @@
       </c>
       <c r="J5" s="7" t="inlineStr">
         <is>
-          <t>-0.111 (t=-0.62)</t>
+          <t>-0.11 (t=-0.62)</t>
         </is>
       </c>
       <c r="K5" s="7" t="inlineStr">
@@ -5105,10 +5105,10 @@
         </is>
       </c>
       <c r="B6" s="21" t="n">
-        <v>48.07</v>
+        <v>47.74</v>
       </c>
       <c r="C6" s="17" t="n">
-        <v>1.98</v>
+        <v>1.95</v>
       </c>
       <c r="D6" s="17" t="n">
         <v>0.059</v>
@@ -5118,27 +5118,27 @@
       </c>
       <c r="F6" s="17" t="inlineStr">
         <is>
-          <t>0.056 (t=0.39)</t>
+          <t>0.059 (t=0.41)</t>
         </is>
       </c>
       <c r="G6" s="17" t="inlineStr">
         <is>
-          <t>-0.116 (t=-0.52)</t>
+          <t>-0.119 (t=-0.54)</t>
         </is>
       </c>
       <c r="H6" s="17" t="inlineStr">
         <is>
-          <t>-0.06 (t=-0.31)</t>
+          <t>-0.059 (t=-0.3)</t>
         </is>
       </c>
       <c r="I6" s="17" t="inlineStr">
         <is>
-          <t>0.241 (t=1.31)</t>
+          <t>0.244 (t=1.32)</t>
         </is>
       </c>
       <c r="J6" s="17" t="inlineStr">
         <is>
-          <t>-0.207 (t=-0.72)</t>
+          <t>-0.208 (t=-0.72)</t>
         </is>
       </c>
       <c r="K6" s="17" t="inlineStr">
@@ -5154,7 +5154,7 @@
         </is>
       </c>
       <c r="B7" s="23" t="n">
-        <v>28.62</v>
+        <v>29.07</v>
       </c>
       <c r="C7" s="7" t="n">
         <v>1.03</v>
@@ -5167,32 +5167,32 @@
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>-0.069 (t=-0.42)</t>
+          <t>-0.073 (t=-0.44)</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
-          <t>-0.004 (t=-0.02)</t>
+          <t>0.001 (t=0.0)</t>
         </is>
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
-          <t>0.235 (t=1.04)</t>
+          <t>0.234 (t=1.03)</t>
         </is>
       </c>
       <c r="I7" s="7" t="inlineStr">
         <is>
-          <t>-0.103 (t=-0.49)</t>
+          <t>-0.106 (t=-0.5)</t>
         </is>
       </c>
       <c r="J7" s="7" t="inlineStr">
         <is>
-          <t>0.022 (t=0.07)</t>
+          <t>0.023 (t=0.07)</t>
         </is>
       </c>
       <c r="K7" s="7" t="inlineStr">
         <is>
-          <t>-0.065 (t=-0.55)</t>
+          <t>-0.064 (t=-0.53)</t>
         </is>
       </c>
     </row>
@@ -5281,10 +5281,10 @@
         </is>
       </c>
       <c r="B4" s="7" t="n">
-        <v>-0.523</v>
+        <v>-0.525</v>
       </c>
       <c r="C4" s="7" t="n">
-        <v>3.81</v>
+        <v>3.836</v>
       </c>
       <c r="D4" s="7" t="n">
         <v>0</v>
@@ -5293,10 +5293,10 @@
         <v>1</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>1.259</v>
+        <v>1.26</v>
       </c>
       <c r="G4" s="7" t="n">
-        <v>1.313</v>
+        <v>1.314</v>
       </c>
       <c r="H4" s="7" t="n">
         <v>0.054</v>
@@ -5309,10 +5309,10 @@
         </is>
       </c>
       <c r="B5" s="17" t="n">
-        <v>-0.416</v>
+        <v>-0.454</v>
       </c>
       <c r="C5" s="17" t="n">
-        <v>2.244</v>
+        <v>2.375</v>
       </c>
       <c r="D5" s="17" t="n">
         <v>0</v>
@@ -5321,13 +5321,13 @@
         <v>1</v>
       </c>
       <c r="F5" s="17" t="n">
-        <v>1.605</v>
+        <v>1.613</v>
       </c>
       <c r="G5" s="17" t="n">
-        <v>1.677</v>
+        <v>1.693</v>
       </c>
       <c r="H5" s="17" t="n">
-        <v>0.07199999999999999</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="6">
@@ -5337,10 +5337,10 @@
         </is>
       </c>
       <c r="B6" s="7" t="n">
-        <v>0.165</v>
+        <v>0.24</v>
       </c>
       <c r="C6" s="7" t="n">
-        <v>12.035</v>
+        <v>12.251</v>
       </c>
       <c r="D6" s="7" t="n">
         <v>0</v>
@@ -5349,10 +5349,10 @@
         <v>1</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>2.513</v>
+        <v>2.526</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>2.513</v>
+        <v>2.526</v>
       </c>
       <c r="H6" s="7" t="n">
         <v>0</v>
@@ -5417,13 +5417,13 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>1.252</v>
+        <v>1.25</v>
       </c>
       <c r="C9" s="7" t="n">
-        <v>0.8213</v>
+        <v>0.8209</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="E9" s="7" t="n">
         <v>8.609999999999999</v>
@@ -5435,13 +5435,13 @@
         <v>77.2</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>6.74</v>
+        <v>6.72</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>3.37</v>
+        <v>3.36</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>3.632</v>
+        <v>5.526</v>
       </c>
     </row>
     <row r="10">
@@ -5451,13 +5451,13 @@
         </is>
       </c>
       <c r="B10" s="17" t="n">
-        <v>1.437</v>
+        <v>1.413</v>
       </c>
       <c r="C10" s="17" t="n">
-        <v>0.8551</v>
+        <v>0.8506</v>
       </c>
       <c r="D10" s="17" t="n">
-        <v>346</v>
+        <v>359</v>
       </c>
       <c r="E10" s="17" t="n">
         <v>8.65</v>
@@ -5469,10 +5469,10 @@
         <v>75.90000000000001</v>
       </c>
       <c r="H10" s="17" t="n">
-        <v>6.91</v>
+        <v>6.74</v>
       </c>
       <c r="I10" s="17" t="n">
-        <v>3.45</v>
+        <v>3.37</v>
       </c>
       <c r="J10" s="17" t="n">
         <v>0.316</v>
@@ -5485,13 +5485,13 @@
         </is>
       </c>
       <c r="B11" s="7" t="n">
-        <v>0.368</v>
+        <v>0.383</v>
       </c>
       <c r="C11" s="7" t="n">
-        <v>0.6092</v>
+        <v>0.6137</v>
       </c>
       <c r="D11" s="7" t="n">
-        <v>5035</v>
+        <v>4639</v>
       </c>
       <c r="E11" s="7" t="n">
         <v>15.04</v>
@@ -5503,13 +5503,13 @@
         <v>80.7</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>0.67</v>
+        <v>0.73</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>0.33</v>
+        <v>0.37</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>8.127000000000001</v>
+        <v>12.559</v>
       </c>
     </row>
   </sheetData>
@@ -5593,7 +5593,7 @@
         <v>0</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>155329.01</v>
+        <v>155150.5</v>
       </c>
     </row>
     <row r="6">
@@ -5622,10 +5622,10 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>2325487.01</v>
+        <v>4228666.25</v>
       </c>
       <c r="C7" s="4" t="n">
-        <v>1534422.46</v>
+        <v>3425427.49</v>
       </c>
       <c r="D7" s="4" t="n">
         <v>1877143.41</v>
@@ -5641,16 +5641,16 @@
         </is>
       </c>
       <c r="B8" s="13" t="n">
-        <v>3676243.11</v>
+        <v>5579422.35</v>
       </c>
       <c r="C8" s="13" t="n">
-        <v>2503433.82</v>
+        <v>4394438.85</v>
       </c>
       <c r="D8" s="13" t="n">
         <v>3443683.26</v>
       </c>
       <c r="E8" s="13" t="n">
-        <v>2120433.21</v>
+        <v>2120254.7</v>
       </c>
     </row>
     <row r="9">
@@ -5679,13 +5679,13 @@
         </is>
       </c>
       <c r="B10" s="13" t="n">
-        <v>1347073.8</v>
+        <v>3250344.25</v>
       </c>
       <c r="C10" s="13" t="n">
-        <v>564075.33</v>
+        <v>2455194.43</v>
       </c>
       <c r="D10" s="13" t="n">
-        <v>910972.4300000001</v>
+        <v>911068.84</v>
       </c>
       <c r="E10" s="15" t="n">
         <v>0</v>
@@ -5698,13 +5698,13 @@
         </is>
       </c>
       <c r="B11" s="4" t="n">
-        <v>2671344.49</v>
+        <v>4574614.94</v>
       </c>
       <c r="C11" s="4" t="n">
-        <v>1514086.47</v>
+        <v>3405205.57</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>2446795.81</v>
+        <v>2446892.22</v>
       </c>
       <c r="E11" s="4" t="n">
         <v>1067096.39</v>
@@ -5717,16 +5717,16 @@
         </is>
       </c>
       <c r="B12" s="13" t="n">
-        <v>1004898.62</v>
+        <v>1004807.41</v>
       </c>
       <c r="C12" s="13" t="n">
-        <v>989347.35</v>
+        <v>989233.28</v>
       </c>
       <c r="D12" s="13" t="n">
-        <v>996887.45</v>
+        <v>996791.04</v>
       </c>
       <c r="E12" s="13" t="n">
-        <v>1053336.82</v>
+        <v>1053158.31</v>
       </c>
     </row>
     <row r="13">
@@ -5736,16 +5736,16 @@
         </is>
       </c>
       <c r="B13" s="7" t="n">
-        <v>3.632</v>
+        <v>5.526</v>
       </c>
       <c r="C13" s="7" t="n">
-        <v>2.511</v>
+        <v>4.423</v>
       </c>
       <c r="D13" s="7" t="n">
         <v>3.424</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>1.845</v>
+        <v>1.846</v>
       </c>
     </row>
     <row r="14">
@@ -5755,10 +5755,10 @@
         </is>
       </c>
       <c r="B14" s="17" t="n">
-        <v>0.996</v>
+        <v>2.89</v>
       </c>
       <c r="C14" s="17" t="n">
-        <v>0.591</v>
+        <v>2.502</v>
       </c>
       <c r="D14" s="17" t="n">
         <v>0.342</v>
@@ -5774,10 +5774,10 @@
         </is>
       </c>
       <c r="B15" s="4" t="n">
-        <v>729951.54</v>
+        <v>1110587.39</v>
       </c>
       <c r="C15" s="4" t="n">
-        <v>496886.72</v>
+        <v>875087.73</v>
       </c>
       <c r="D15" s="4" t="n">
         <v>682593.36</v>
@@ -5792,17 +5792,17 @@
           <t>Excess Liquidity 超额流动性</t>
         </is>
       </c>
-      <c r="B16" s="13" t="n">
-        <v>274947.08</v>
+      <c r="B16" s="18" t="n">
+        <v>-105779.98</v>
       </c>
       <c r="C16" s="13" t="n">
-        <v>492460.63</v>
+        <v>114145.55</v>
       </c>
       <c r="D16" s="13" t="n">
-        <v>314294.09</v>
+        <v>314197.68</v>
       </c>
       <c r="E16" s="13" t="n">
-        <v>664584.37</v>
+        <v>664405.86</v>
       </c>
     </row>
     <row r="17">
@@ -5815,7 +5815,7 @@
         <v>0</v>
       </c>
       <c r="C17" s="7" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="D17" s="7" t="n">
         <v>0</v>
@@ -5865,13 +5865,13 @@
         </is>
       </c>
       <c r="B21" s="4" t="n">
-        <v>1004898.62</v>
+        <v>1004807.41</v>
       </c>
       <c r="C21" s="4" t="n">
-        <v>989347.35</v>
+        <v>989233.28</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>996887.45</v>
+        <v>996791.04</v>
       </c>
       <c r="E21" s="4" t="n">
         <v>876665.88</v>
@@ -5903,10 +5903,10 @@
         </is>
       </c>
       <c r="B23" s="4" t="n">
-        <v>2325487.01</v>
+        <v>4228666.25</v>
       </c>
       <c r="C23" s="4" t="n">
-        <v>1534422.46</v>
+        <v>3425427.49</v>
       </c>
       <c r="D23" s="4" t="n">
         <v>1877143.41</v>
@@ -5922,13 +5922,13 @@
         </is>
       </c>
       <c r="B24" s="13" t="n">
-        <v>1320588.39</v>
+        <v>3223858.84</v>
       </c>
       <c r="C24" s="13" t="n">
-        <v>545075.11</v>
+        <v>2436194.21</v>
       </c>
       <c r="D24" s="13" t="n">
-        <v>880255.96</v>
+        <v>880352.37</v>
       </c>
       <c r="E24" s="15" t="n">
         <v>0</v>
@@ -5941,13 +5941,13 @@
         </is>
       </c>
       <c r="B25" s="4" t="n">
-        <v>1004898.62</v>
+        <v>1004807.41</v>
       </c>
       <c r="C25" s="4" t="n">
-        <v>989347.35</v>
+        <v>989233.28</v>
       </c>
       <c r="D25" s="4" t="n">
-        <v>996887.45</v>
+        <v>996791.04</v>
       </c>
       <c r="E25" s="4" t="n">
         <v>876665.88</v>
@@ -6083,7 +6083,7 @@
         <v>0</v>
       </c>
       <c r="E32" s="13" t="n">
-        <v>155329.01</v>
+        <v>155150.5</v>
       </c>
     </row>
     <row r="33">
@@ -6093,16 +6093,16 @@
         </is>
       </c>
       <c r="B33" s="4" t="n">
-        <v>1004898.62</v>
+        <v>1004807.41</v>
       </c>
       <c r="C33" s="4" t="n">
-        <v>989347.35</v>
+        <v>989233.28</v>
       </c>
       <c r="D33" s="4" t="n">
-        <v>996887.45</v>
+        <v>996791.04</v>
       </c>
       <c r="E33" s="4" t="n">
-        <v>1053336.82</v>
+        <v>1053158.31</v>
       </c>
     </row>
     <row r="34">
@@ -6165,16 +6165,16 @@
         </is>
       </c>
       <c r="B39" s="4" t="n">
-        <v>479492.41</v>
+        <v>478446.74</v>
       </c>
       <c r="C39" s="4" t="n">
-        <v>420303.88</v>
+        <v>419263.54</v>
       </c>
       <c r="D39" s="4" t="n">
-        <v>249710.29</v>
+        <v>248670.31</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>426377.54</v>
+        <v>425244.41</v>
       </c>
     </row>
     <row r="40">
@@ -6222,16 +6222,16 @@
         </is>
       </c>
       <c r="B42" s="13" t="n">
-        <v>663803.38</v>
+        <v>662757.71</v>
       </c>
       <c r="C42" s="13" t="n">
-        <v>724040.99</v>
+        <v>723000.65</v>
       </c>
       <c r="D42" s="13" t="n">
-        <v>980263.26</v>
+        <v>979223.28</v>
       </c>
       <c r="E42" s="13" t="n">
-        <v>823644.49</v>
+        <v>822511.36</v>
       </c>
     </row>
     <row r="43">
@@ -6298,16 +6298,16 @@
         </is>
       </c>
       <c r="B46" s="13" t="n">
-        <v>578256.1</v>
+        <v>577210.4300000001</v>
       </c>
       <c r="C46" s="13" t="n">
-        <v>575306.51</v>
+        <v>574266.17</v>
       </c>
       <c r="D46" s="13" t="n">
-        <v>575110.5699999999</v>
+        <v>574070.59</v>
       </c>
       <c r="E46" s="13" t="n">
-        <v>626622.02</v>
+        <v>625488.89</v>
       </c>
     </row>
     <row r="47">
@@ -6320,13 +6320,13 @@
         <v>0.316</v>
       </c>
       <c r="C47" s="7" t="n">
-        <v>0.523</v>
+        <v>0.524</v>
       </c>
       <c r="D47" s="7" t="n">
-        <v>1.256</v>
+        <v>1.258</v>
       </c>
       <c r="E47" s="7" t="n">
-        <v>0.628</v>
+        <v>0.629</v>
       </c>
     </row>
     <row r="48">
@@ -6374,16 +6374,16 @@
         </is>
       </c>
       <c r="B50" s="13" t="n">
-        <v>541736.1</v>
+        <v>540690.4300000001</v>
       </c>
       <c r="C50" s="13" t="n">
-        <v>515154.03</v>
+        <v>514113.69</v>
       </c>
       <c r="D50" s="13" t="n">
-        <v>430620.59</v>
+        <v>429580.61</v>
       </c>
       <c r="E50" s="13" t="n">
-        <v>547956.72</v>
+        <v>546823.59</v>
       </c>
     </row>
     <row r="51">
@@ -6402,7 +6402,7 @@
         <v>0</v>
       </c>
       <c r="E51" s="7" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
     </row>
     <row r="53">
@@ -6655,16 +6655,16 @@
         </is>
       </c>
       <c r="B66" s="13" t="n">
-        <v>479492.41</v>
+        <v>478446.74</v>
       </c>
       <c r="C66" s="13" t="n">
-        <v>420303.88</v>
+        <v>419263.54</v>
       </c>
       <c r="D66" s="13" t="n">
-        <v>249710.29</v>
+        <v>248670.31</v>
       </c>
       <c r="E66" s="13" t="n">
-        <v>426377.54</v>
+        <v>425244.41</v>
       </c>
     </row>
     <row r="67">
@@ -6674,16 +6674,16 @@
         </is>
       </c>
       <c r="B67" s="4" t="n">
-        <v>578256.1</v>
+        <v>577210.4300000001</v>
       </c>
       <c r="C67" s="4" t="n">
-        <v>575306.51</v>
+        <v>574266.17</v>
       </c>
       <c r="D67" s="4" t="n">
-        <v>575110.5699999999</v>
+        <v>574070.59</v>
       </c>
       <c r="E67" s="4" t="n">
-        <v>626622.02</v>
+        <v>625488.89</v>
       </c>
     </row>
     <row r="68">
@@ -6784,10 +6784,10 @@
         </is>
       </c>
       <c r="B75" s="4" t="n">
-        <v>2228434.27</v>
+        <v>4131613.51</v>
       </c>
       <c r="C75" s="4" t="n">
-        <v>1382394.52</v>
+        <v>3273399.55</v>
       </c>
       <c r="D75" s="4" t="n">
         <v>1559846.18</v>
@@ -6803,10 +6803,10 @@
         </is>
       </c>
       <c r="B76" s="13" t="n">
-        <v>3491932.15</v>
+        <v>5395111.39</v>
       </c>
       <c r="C76" s="13" t="n">
-        <v>2199696.71</v>
+        <v>4090701.74</v>
       </c>
       <c r="D76" s="13" t="n">
         <v>2713130.28</v>
@@ -6841,16 +6841,16 @@
         </is>
       </c>
       <c r="B78" s="13" t="n">
-        <v>1826566.22</v>
+        <v>3728791</v>
       </c>
       <c r="C78" s="13" t="n">
-        <v>984379.21</v>
+        <v>2874457.97</v>
       </c>
       <c r="D78" s="13" t="n">
-        <v>1160682.71</v>
+        <v>1159739.14</v>
       </c>
       <c r="E78" s="13" t="n">
-        <v>271048.54</v>
+        <v>270093.92</v>
       </c>
     </row>
     <row r="79">
@@ -6860,16 +6860,16 @@
         </is>
       </c>
       <c r="B79" s="4" t="n">
-        <v>3065289.63</v>
+        <v>4967514.41</v>
       </c>
       <c r="C79" s="4" t="n">
-        <v>1785655.87</v>
+        <v>3675734.63</v>
       </c>
       <c r="D79" s="4" t="n">
-        <v>2291353.4</v>
+        <v>2290409.83</v>
       </c>
       <c r="E79" s="4" t="n">
-        <v>1141122.45</v>
+        <v>1140167.83</v>
       </c>
     </row>
     <row r="80">
@@ -6879,16 +6879,16 @@
         </is>
       </c>
       <c r="B80" s="13" t="n">
-        <v>426642.52</v>
+        <v>427596.98</v>
       </c>
       <c r="C80" s="13" t="n">
-        <v>414040.84</v>
+        <v>414967.11</v>
       </c>
       <c r="D80" s="13" t="n">
-        <v>421776.88</v>
+        <v>422720.45</v>
       </c>
       <c r="E80" s="13" t="n">
-        <v>426714.8</v>
+        <v>427669.42</v>
       </c>
     </row>
     <row r="81">
@@ -6898,16 +6898,16 @@
         </is>
       </c>
       <c r="B81" s="7" t="n">
-        <v>8.127000000000001</v>
+        <v>12.559</v>
       </c>
       <c r="C81" s="7" t="n">
-        <v>5.274</v>
+        <v>9.819000000000001</v>
       </c>
       <c r="D81" s="7" t="n">
-        <v>6.379</v>
+        <v>6.365</v>
       </c>
       <c r="E81" s="7" t="n">
-        <v>3.633</v>
+        <v>3.625</v>
       </c>
     </row>
     <row r="82">
@@ -6917,16 +6917,16 @@
         </is>
       </c>
       <c r="B82" s="17" t="n">
-        <v>2.32</v>
+        <v>6.765</v>
       </c>
       <c r="C82" s="17" t="n">
-        <v>1.404</v>
+        <v>5.957</v>
       </c>
       <c r="D82" s="17" t="n">
-        <v>1.018</v>
+        <v>1.015</v>
       </c>
       <c r="E82" s="17" t="n">
-        <v>-0.445</v>
+        <v>-0.444</v>
       </c>
     </row>
     <row r="83">
@@ -6936,10 +6936,10 @@
         </is>
       </c>
       <c r="B83" s="4" t="n">
-        <v>693431.54</v>
+        <v>1074067.38</v>
       </c>
       <c r="C83" s="4" t="n">
-        <v>436734.24</v>
+        <v>814935.24</v>
       </c>
       <c r="D83" s="4" t="n">
         <v>538103.37</v>
@@ -6955,16 +6955,16 @@
         </is>
       </c>
       <c r="B84" s="18" t="n">
-        <v>-266789.02</v>
+        <v>-646470.4</v>
       </c>
       <c r="C84" s="18" t="n">
-        <v>-22693.4</v>
+        <v>-399968.13</v>
       </c>
       <c r="D84" s="18" t="n">
-        <v>-116326.49</v>
+        <v>-115382.92</v>
       </c>
       <c r="E84" s="13" t="n">
-        <v>116627.65</v>
+        <v>117582.27</v>
       </c>
     </row>
     <row r="85">
@@ -6974,7 +6974,7 @@
         </is>
       </c>
       <c r="B85" s="7" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="C85" s="7" t="n">
         <v>0</v>
@@ -6983,7 +6983,7 @@
         <v>-0</v>
       </c>
       <c r="E85" s="7" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
     </row>
     <row r="87">
@@ -7027,16 +7027,16 @@
         </is>
       </c>
       <c r="B89" s="4" t="n">
-        <v>426642.52</v>
+        <v>427596.98</v>
       </c>
       <c r="C89" s="4" t="n">
-        <v>414040.84</v>
+        <v>414967.11</v>
       </c>
       <c r="D89" s="4" t="n">
-        <v>421776.88</v>
+        <v>422720.45</v>
       </c>
       <c r="E89" s="4" t="n">
-        <v>426714.8</v>
+        <v>427669.42</v>
       </c>
     </row>
     <row r="90">
@@ -7065,10 +7065,10 @@
         </is>
       </c>
       <c r="B91" s="4" t="n">
-        <v>2228434.27</v>
+        <v>4131613.51</v>
       </c>
       <c r="C91" s="4" t="n">
-        <v>1382394.52</v>
+        <v>3273399.55</v>
       </c>
       <c r="D91" s="4" t="n">
         <v>1559846.18</v>
@@ -7084,16 +7084,16 @@
         </is>
       </c>
       <c r="B92" s="13" t="n">
-        <v>1801791.75</v>
+        <v>3704016.53</v>
       </c>
       <c r="C92" s="13" t="n">
-        <v>968353.6800000001</v>
+        <v>2858432.44</v>
       </c>
       <c r="D92" s="13" t="n">
-        <v>1138069.3</v>
+        <v>1137125.73</v>
       </c>
       <c r="E92" s="13" t="n">
-        <v>253647.06</v>
+        <v>252692.44</v>
       </c>
     </row>
     <row r="93">
@@ -7103,16 +7103,16 @@
         </is>
       </c>
       <c r="B93" s="4" t="n">
-        <v>426642.52</v>
+        <v>427596.98</v>
       </c>
       <c r="C93" s="4" t="n">
-        <v>414040.84</v>
+        <v>414967.11</v>
       </c>
       <c r="D93" s="4" t="n">
-        <v>421776.88</v>
+        <v>422720.45</v>
       </c>
       <c r="E93" s="4" t="n">
-        <v>426714.8</v>
+        <v>427669.42</v>
       </c>
     </row>
     <row r="94">
@@ -7239,7 +7239,7 @@
         <v>0</v>
       </c>
       <c r="C100" s="15" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="D100" s="15" t="n">
         <v>0</v>
@@ -7255,16 +7255,16 @@
         </is>
       </c>
       <c r="B101" s="4" t="n">
-        <v>426642.52</v>
+        <v>427596.98</v>
       </c>
       <c r="C101" s="4" t="n">
-        <v>414040.84</v>
+        <v>414967.11</v>
       </c>
       <c r="D101" s="4" t="n">
-        <v>421776.88</v>
+        <v>422720.45</v>
       </c>
       <c r="E101" s="4" t="n">
-        <v>426714.8</v>
+        <v>427669.42</v>
       </c>
     </row>
     <row r="102">
@@ -7358,16 +7358,16 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>15551.27</v>
+        <v>15574.13</v>
       </c>
       <c r="C5" s="4" t="n">
-        <v>8011.17</v>
+        <v>8016.37</v>
       </c>
       <c r="D5" s="19" t="n">
-        <v>-48438.2</v>
+        <v>-48350.9</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>83399.83</v>
+        <v>83308.62</v>
       </c>
     </row>
     <row r="6">
@@ -7377,16 +7377,16 @@
         </is>
       </c>
       <c r="B6" s="13" t="n">
-        <v>184.53</v>
+        <v>445.25</v>
       </c>
       <c r="C6" s="13" t="n">
-        <v>922.65</v>
+        <v>2226.26</v>
       </c>
       <c r="D6" s="13" t="n">
-        <v>3875.14</v>
+        <v>9350.309999999999</v>
       </c>
       <c r="E6" s="13" t="n">
-        <v>26756.95</v>
+        <v>64561.63</v>
       </c>
     </row>
     <row r="7">
@@ -7396,7 +7396,7 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>97984.31</v>
+        <v>2001163.55</v>
       </c>
     </row>
     <row r="9">
@@ -7440,16 +7440,16 @@
         </is>
       </c>
       <c r="B11" s="4" t="n">
-        <v>2949.59</v>
+        <v>2944.26</v>
       </c>
       <c r="C11" s="4" t="n">
-        <v>3145.53</v>
+        <v>3139.84</v>
       </c>
       <c r="D11" s="19" t="n">
-        <v>-48365.92</v>
+        <v>-48278.46</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>68924.16</v>
+        <v>67878.49000000001</v>
       </c>
     </row>
     <row r="12">
@@ -7522,16 +7522,16 @@
         </is>
       </c>
       <c r="B17" s="4" t="n">
-        <v>12601.68</v>
+        <v>12629.87</v>
       </c>
       <c r="C17" s="4" t="n">
-        <v>4865.64</v>
+        <v>4876.53</v>
       </c>
       <c r="D17" s="20" t="n">
-        <v>-72.28</v>
+        <v>-72.44</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>14475.67</v>
+        <v>15430.13</v>
       </c>
     </row>
     <row r="18">
@@ -7541,16 +7541,16 @@
         </is>
       </c>
       <c r="B18" s="13" t="n">
-        <v>250.21</v>
+        <v>510.79</v>
       </c>
       <c r="C18" s="13" t="n">
-        <v>1251.07</v>
+        <v>2553.97</v>
       </c>
       <c r="D18" s="13" t="n">
-        <v>5254.51</v>
+        <v>10726.66</v>
       </c>
       <c r="E18" s="13" t="n">
-        <v>36281.11</v>
+        <v>74065.03</v>
       </c>
     </row>
     <row r="19">
@@ -7560,7 +7560,7 @@
         </is>
       </c>
       <c r="B19" s="4" t="n">
-        <v>84728.47</v>
+        <v>1987907.71</v>
       </c>
     </row>
     <row r="21">
@@ -7642,13 +7642,13 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>989347.35</v>
+        <v>989233.28</v>
       </c>
       <c r="C5" s="4" t="n">
-        <v>996887.45</v>
+        <v>996791.04</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>1053336.82</v>
+        <v>1053158.31</v>
       </c>
       <c r="E5" s="4" t="n">
         <v>921498.79</v>
@@ -7661,16 +7661,16 @@
         </is>
       </c>
       <c r="B6" s="13" t="n">
-        <v>15551.27</v>
+        <v>15574.13</v>
       </c>
       <c r="C6" s="13" t="n">
-        <v>8011.17</v>
+        <v>8016.37</v>
       </c>
       <c r="D6" s="18" t="n">
-        <v>-48438.2</v>
+        <v>-48350.9</v>
       </c>
       <c r="E6" s="13" t="n">
-        <v>83399.83</v>
+        <v>83308.62</v>
       </c>
     </row>
     <row r="7">
@@ -7718,16 +7718,16 @@
         </is>
       </c>
       <c r="B9" s="4" t="n">
-        <v>1004898.62</v>
+        <v>1004807.41</v>
       </c>
       <c r="C9" s="4" t="n">
-        <v>1004898.62</v>
+        <v>1004807.41</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>1004898.62</v>
+        <v>1004807.41</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>1004898.62</v>
+        <v>1004807.41</v>
       </c>
     </row>
     <row r="10">
@@ -7743,10 +7743,10 @@
         <v>0.8</v>
       </c>
       <c r="D10" s="22" t="n">
-        <v>-4.6</v>
+        <v>-4.59</v>
       </c>
       <c r="E10" s="21" t="n">
-        <v>9.050000000000001</v>
+        <v>9.039999999999999</v>
       </c>
     </row>
     <row r="11">
@@ -7759,7 +7759,7 @@
         <v>0</v>
       </c>
       <c r="C11" s="24" t="n">
-        <v>-2.68</v>
+        <v>-2.69</v>
       </c>
       <c r="D11" s="24" t="n">
         <v>-6.07</v>
@@ -7809,13 +7809,13 @@
         </is>
       </c>
       <c r="B15" s="4" t="n">
-        <v>575306.51</v>
+        <v>574266.17</v>
       </c>
       <c r="C15" s="4" t="n">
-        <v>575110.5699999999</v>
+        <v>574070.59</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>626622.02</v>
+        <v>625488.89</v>
       </c>
       <c r="E15" s="4" t="n">
         <v>509331.94</v>
@@ -7828,16 +7828,16 @@
         </is>
       </c>
       <c r="B16" s="13" t="n">
-        <v>2949.59</v>
+        <v>2944.26</v>
       </c>
       <c r="C16" s="13" t="n">
-        <v>3145.53</v>
+        <v>3139.84</v>
       </c>
       <c r="D16" s="18" t="n">
-        <v>-48365.92</v>
+        <v>-48278.46</v>
       </c>
       <c r="E16" s="13" t="n">
-        <v>68924.16</v>
+        <v>67878.49000000001</v>
       </c>
     </row>
     <row r="17">
@@ -7885,16 +7885,16 @@
         </is>
       </c>
       <c r="B19" s="4" t="n">
-        <v>578256.1</v>
+        <v>577210.4300000001</v>
       </c>
       <c r="C19" s="4" t="n">
-        <v>578256.1</v>
+        <v>577210.4300000001</v>
       </c>
       <c r="D19" s="4" t="n">
-        <v>578256.1</v>
+        <v>577210.4300000001</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>578256.1</v>
+        <v>577210.4300000001</v>
       </c>
     </row>
     <row r="20">
@@ -7913,7 +7913,7 @@
         <v>-7.72</v>
       </c>
       <c r="E20" s="21" t="n">
-        <v>13.53</v>
+        <v>13.33</v>
       </c>
     </row>
     <row r="21">
@@ -7976,13 +7976,13 @@
         </is>
       </c>
       <c r="B25" s="4" t="n">
-        <v>414040.84</v>
+        <v>414967.11</v>
       </c>
       <c r="C25" s="4" t="n">
-        <v>421776.88</v>
+        <v>422720.45</v>
       </c>
       <c r="D25" s="4" t="n">
-        <v>426714.8</v>
+        <v>427669.42</v>
       </c>
       <c r="E25" s="4" t="n">
         <v>412166.85</v>
@@ -7995,16 +7995,16 @@
         </is>
       </c>
       <c r="B26" s="13" t="n">
-        <v>12601.68</v>
+        <v>12629.87</v>
       </c>
       <c r="C26" s="13" t="n">
-        <v>4865.64</v>
+        <v>4876.53</v>
       </c>
       <c r="D26" s="25" t="n">
-        <v>-72.28</v>
+        <v>-72.44</v>
       </c>
       <c r="E26" s="13" t="n">
-        <v>14475.67</v>
+        <v>15430.13</v>
       </c>
     </row>
     <row r="27">
@@ -8052,16 +8052,16 @@
         </is>
       </c>
       <c r="B29" s="4" t="n">
-        <v>426642.52</v>
+        <v>427596.98</v>
       </c>
       <c r="C29" s="4" t="n">
-        <v>426642.52</v>
+        <v>427596.98</v>
       </c>
       <c r="D29" s="4" t="n">
-        <v>426642.52</v>
+        <v>427596.98</v>
       </c>
       <c r="E29" s="4" t="n">
-        <v>426642.52</v>
+        <v>427596.98</v>
       </c>
     </row>
     <row r="30">
@@ -8080,7 +8080,7 @@
         <v>-0.02</v>
       </c>
       <c r="E30" s="21" t="n">
-        <v>3.51</v>
+        <v>3.74</v>
       </c>
     </row>
     <row r="31">
@@ -8149,7 +8149,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>8011.17</v>
+        <v>8016.37</v>
       </c>
     </row>
     <row r="5">
@@ -8159,7 +8159,7 @@
         </is>
       </c>
       <c r="B5" s="19" t="n">
-        <v>-659896.29</v>
+        <v>-2563075.53</v>
       </c>
     </row>
     <row r="6">
@@ -8169,7 +8169,7 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>436101.37</v>
+        <v>2339275.41</v>
       </c>
     </row>
     <row r="7">
@@ -9176,7 +9176,7 @@
         </is>
       </c>
       <c r="B96" s="4" t="n">
-        <v>1011218.51</v>
+        <v>1011202.12</v>
       </c>
     </row>
     <row r="97">
@@ -9186,7 +9186,7 @@
         </is>
       </c>
       <c r="B97" s="13" t="n">
-        <v>1025407</v>
+        <v>1025356.19</v>
       </c>
     </row>
     <row r="98">
@@ -9196,7 +9196,7 @@
         </is>
       </c>
       <c r="B98" s="4" t="n">
-        <v>1026941.31</v>
+        <v>1026905.51</v>
       </c>
     </row>
     <row r="99">
@@ -9206,7 +9206,7 @@
         </is>
       </c>
       <c r="B99" s="13" t="n">
-        <v>1015258.85</v>
+        <v>1015273.3</v>
       </c>
     </row>
     <row r="100">
@@ -9216,7 +9216,7 @@
         </is>
       </c>
       <c r="B100" s="4" t="n">
-        <v>1003003.03</v>
+        <v>1003025.8</v>
       </c>
     </row>
     <row r="101">
@@ -9226,7 +9226,7 @@
         </is>
       </c>
       <c r="B101" s="13" t="n">
-        <v>1013068.4</v>
+        <v>1013098.34</v>
       </c>
     </row>
     <row r="102">
@@ -9236,7 +9236,7 @@
         </is>
       </c>
       <c r="B102" s="4" t="n">
-        <v>1026667.89</v>
+        <v>1026718.34</v>
       </c>
     </row>
     <row r="103">
@@ -9246,7 +9246,7 @@
         </is>
       </c>
       <c r="B103" s="13" t="n">
-        <v>1053397.75</v>
+        <v>1053504.94</v>
       </c>
     </row>
     <row r="104">
@@ -9256,7 +9256,7 @@
         </is>
       </c>
       <c r="B104" s="4" t="n">
-        <v>1050736.08</v>
+        <v>1050844.96</v>
       </c>
     </row>
     <row r="105">
@@ -9266,7 +9266,7 @@
         </is>
       </c>
       <c r="B105" s="13" t="n">
-        <v>1049499.07</v>
+        <v>1049581.91</v>
       </c>
     </row>
     <row r="106">
@@ -9276,7 +9276,7 @@
         </is>
       </c>
       <c r="B106" s="4" t="n">
-        <v>1049134.93</v>
+        <v>1049200.21</v>
       </c>
     </row>
     <row r="107">
@@ -9286,7 +9286,7 @@
         </is>
       </c>
       <c r="B107" s="13" t="n">
-        <v>1042919.9</v>
+        <v>1042965.78</v>
       </c>
     </row>
     <row r="108">
@@ -9296,7 +9296,7 @@
         </is>
       </c>
       <c r="B108" s="4" t="n">
-        <v>1048685.92</v>
+        <v>1048734.43</v>
       </c>
     </row>
     <row r="109">
@@ -9306,7 +9306,7 @@
         </is>
       </c>
       <c r="B109" s="13" t="n">
-        <v>1042773.4</v>
+        <v>1042822.5</v>
       </c>
     </row>
     <row r="110">
@@ -9316,7 +9316,7 @@
         </is>
       </c>
       <c r="B110" s="4" t="n">
-        <v>1044235.83</v>
+        <v>1044292.9</v>
       </c>
     </row>
     <row r="111">
@@ -9326,7 +9326,7 @@
         </is>
       </c>
       <c r="B111" s="13" t="n">
-        <v>1070354.14</v>
+        <v>1070408.83</v>
       </c>
     </row>
     <row r="112">
@@ -9336,7 +9336,7 @@
         </is>
       </c>
       <c r="B112" s="4" t="n">
-        <v>1061514.84</v>
+        <v>1061559.43</v>
       </c>
     </row>
     <row r="113">
@@ -9346,7 +9346,7 @@
         </is>
       </c>
       <c r="B113" s="13" t="n">
-        <v>1074870.62</v>
+        <v>1074879.59</v>
       </c>
     </row>
     <row r="114">
@@ -9356,7 +9356,7 @@
         </is>
       </c>
       <c r="B114" s="4" t="n">
-        <v>1080512.52</v>
+        <v>1080503.54</v>
       </c>
     </row>
     <row r="115">
@@ -9366,7 +9366,7 @@
         </is>
       </c>
       <c r="B115" s="13" t="n">
-        <v>1086924.48</v>
+        <v>1086894.67</v>
       </c>
     </row>
     <row r="116">
@@ -9376,7 +9376,7 @@
         </is>
       </c>
       <c r="B116" s="4" t="n">
-        <v>1071780.32</v>
+        <v>1071796.37</v>
       </c>
     </row>
     <row r="117">
@@ -9386,7 +9386,7 @@
         </is>
       </c>
       <c r="B117" s="13" t="n">
-        <v>1065526.09</v>
+        <v>1065522.69</v>
       </c>
     </row>
     <row r="118">
@@ -9396,7 +9396,7 @@
         </is>
       </c>
       <c r="B118" s="4" t="n">
-        <v>1080594.32</v>
+        <v>1080563.67</v>
       </c>
     </row>
     <row r="119">
@@ -9406,7 +9406,7 @@
         </is>
       </c>
       <c r="B119" s="13" t="n">
-        <v>1075591.99</v>
+        <v>1075540.76</v>
       </c>
     </row>
     <row r="120">
@@ -9416,7 +9416,7 @@
         </is>
       </c>
       <c r="B120" s="4" t="n">
-        <v>1071013.67</v>
+        <v>1070952.2</v>
       </c>
     </row>
     <row r="121">
@@ -9426,7 +9426,7 @@
         </is>
       </c>
       <c r="B121" s="13" t="n">
-        <v>1073689.47</v>
+        <v>1073612.17</v>
       </c>
     </row>
     <row r="122">
@@ -9436,7 +9436,7 @@
         </is>
       </c>
       <c r="B122" s="4" t="n">
-        <v>1074236.64</v>
+        <v>1074160.56</v>
       </c>
     </row>
     <row r="123">
@@ -9446,7 +9446,7 @@
         </is>
       </c>
       <c r="B123" s="13" t="n">
-        <v>1084547.15</v>
+        <v>1084460.75</v>
       </c>
     </row>
     <row r="124">
@@ -9456,7 +9456,7 @@
         </is>
       </c>
       <c r="B124" s="4" t="n">
-        <v>1085528.37</v>
+        <v>1085444.17</v>
       </c>
     </row>
     <row r="125">
@@ -9466,7 +9466,7 @@
         </is>
       </c>
       <c r="B125" s="13" t="n">
-        <v>1092616.33</v>
+        <v>1092531.84</v>
       </c>
     </row>
     <row r="126">
@@ -9476,7 +9476,7 @@
         </is>
       </c>
       <c r="B126" s="4" t="n">
-        <v>1092781.06</v>
+        <v>1092690.79</v>
       </c>
     </row>
     <row r="127">
@@ -9486,7 +9486,7 @@
         </is>
       </c>
       <c r="B127" s="13" t="n">
-        <v>1053336.82</v>
+        <v>1053158.31</v>
       </c>
     </row>
     <row r="128">
@@ -9496,7 +9496,7 @@
         </is>
       </c>
       <c r="B128" s="4" t="n">
-        <v>1049687.33</v>
+        <v>1049512.64</v>
       </c>
     </row>
     <row r="129">
@@ -9506,7 +9506,7 @@
         </is>
       </c>
       <c r="B129" s="13" t="n">
-        <v>1044100.12</v>
+        <v>1043936.06</v>
       </c>
     </row>
     <row r="130">
@@ -9516,7 +9516,7 @@
         </is>
       </c>
       <c r="B130" s="4" t="n">
-        <v>1032626.83</v>
+        <v>1032472.74</v>
       </c>
     </row>
     <row r="131">
@@ -9526,7 +9526,7 @@
         </is>
       </c>
       <c r="B131" s="13" t="n">
-        <v>1039700.39</v>
+        <v>1039556.14</v>
       </c>
     </row>
     <row r="132">
@@ -9536,7 +9536,7 @@
         </is>
       </c>
       <c r="B132" s="4" t="n">
-        <v>1037551.62</v>
+        <v>1037415.03</v>
       </c>
     </row>
     <row r="133">
@@ -9546,7 +9546,7 @@
         </is>
       </c>
       <c r="B133" s="13" t="n">
-        <v>1019311.74</v>
+        <v>1019194.66</v>
       </c>
     </row>
     <row r="134">
@@ -9556,7 +9556,7 @@
         </is>
       </c>
       <c r="B134" s="4" t="n">
-        <v>1014163.76</v>
+        <v>1014068.88</v>
       </c>
     </row>
     <row r="135">
@@ -9566,7 +9566,7 @@
         </is>
       </c>
       <c r="B135" s="13" t="n">
-        <v>999293.04</v>
+        <v>999221.6800000001</v>
       </c>
     </row>
     <row r="136">
@@ -9576,7 +9576,7 @@
         </is>
       </c>
       <c r="B136" s="4" t="n">
-        <v>1011409.78</v>
+        <v>1011311.18</v>
       </c>
     </row>
     <row r="137">
@@ -9586,7 +9586,7 @@
         </is>
       </c>
       <c r="B137" s="13" t="n">
-        <v>1014540.8</v>
+        <v>1014433.88</v>
       </c>
     </row>
     <row r="138">
@@ -9596,7 +9596,7 @@
         </is>
       </c>
       <c r="B138" s="4" t="n">
-        <v>1011881.11</v>
+        <v>1011774.92</v>
       </c>
     </row>
     <row r="139">
@@ -9606,7 +9606,7 @@
         </is>
       </c>
       <c r="B139" s="13" t="n">
-        <v>998415.39</v>
+        <v>998320.26</v>
       </c>
     </row>
     <row r="140">
@@ -9616,7 +9616,7 @@
         </is>
       </c>
       <c r="B140" s="4" t="n">
-        <v>1014351.76</v>
+        <v>1014291.81</v>
       </c>
     </row>
     <row r="141">
@@ -9626,7 +9626,7 @@
         </is>
       </c>
       <c r="B141" s="13" t="n">
-        <v>1023498.77</v>
+        <v>1023430.49</v>
       </c>
     </row>
     <row r="142">
@@ -9636,7 +9636,7 @@
         </is>
       </c>
       <c r="B142" s="4" t="n">
-        <v>1023696.66</v>
+        <v>1023647.26</v>
       </c>
     </row>
     <row r="143">
@@ -9646,7 +9646,7 @@
         </is>
       </c>
       <c r="B143" s="13" t="n">
-        <v>996887.45</v>
+        <v>996791.04</v>
       </c>
     </row>
     <row r="144">
@@ -9656,7 +9656,7 @@
         </is>
       </c>
       <c r="B144" s="4" t="n">
-        <v>1016573.57</v>
+        <v>1016545.25</v>
       </c>
     </row>
     <row r="145">
@@ -9666,7 +9666,7 @@
         </is>
       </c>
       <c r="B145" s="13" t="n">
-        <v>997861.24</v>
+        <v>997800.67</v>
       </c>
     </row>
     <row r="146">
@@ -9676,7 +9676,7 @@
         </is>
       </c>
       <c r="B146" s="4" t="n">
-        <v>991493.7</v>
+        <v>991400.37</v>
       </c>
     </row>
     <row r="147">
@@ -9686,7 +9686,7 @@
         </is>
       </c>
       <c r="B147" s="13" t="n">
-        <v>989347.35</v>
+        <v>989233.28</v>
       </c>
     </row>
     <row r="148">
@@ -9696,7 +9696,7 @@
         </is>
       </c>
       <c r="B148" s="4" t="n">
-        <v>1004898.62</v>
+        <v>1004807.41</v>
       </c>
     </row>
   </sheetData>
@@ -9801,31 +9801,31 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>1004898.62</v>
+        <v>1004807.41</v>
       </c>
       <c r="C4" s="4" t="n">
-        <v>2325487.01</v>
+        <v>4228666.25</v>
       </c>
       <c r="D4" s="4" t="n">
         <v>1324270.69</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>3649757.7</v>
+        <v>5552936.94</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>1001216.32</v>
+        <v>2904395.56</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>3.632</v>
+        <v>5.526</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>0.996</v>
+        <v>2.89</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>363.2</v>
+        <v>552.64</v>
       </c>
       <c r="J4" s="5" t="n">
-        <v>181.6</v>
+        <v>276.32</v>
       </c>
       <c r="K4" s="26" t="n">
         <v>19</v>
@@ -9838,7 +9838,7 @@
         </is>
       </c>
       <c r="B5" s="13" t="n">
-        <v>578256.1</v>
+        <v>577210.4300000001</v>
       </c>
       <c r="C5" s="13" t="n">
         <v>97052.74000000001</v>
@@ -9859,10 +9859,10 @@
         <v>0.02</v>
       </c>
       <c r="I5" s="27" t="n">
-        <v>31.58</v>
+        <v>31.63</v>
       </c>
       <c r="J5" s="27" t="n">
-        <v>15.79</v>
+        <v>15.82</v>
       </c>
       <c r="K5" s="28" t="n">
         <v>1</v>
@@ -9875,31 +9875,31 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>426642.52</v>
+        <v>427596.98</v>
       </c>
       <c r="C6" s="4" t="n">
-        <v>2228434.27</v>
+        <v>4131613.51</v>
       </c>
       <c r="D6" s="4" t="n">
         <v>1238723.41</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>3467157.68</v>
+        <v>5370336.92</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>989710.86</v>
+        <v>2892890.1</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>8.127000000000001</v>
+        <v>12.559</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>2.32</v>
+        <v>6.765</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>812.66</v>
+        <v>1255.93</v>
       </c>
       <c r="J6" s="5" t="n">
-        <v>406.33</v>
+        <v>627.97</v>
       </c>
       <c r="K6" s="26" t="n">
         <v>18</v>
@@ -9940,7 +9940,7 @@
     <row r="3">
       <c r="A3" s="29" t="inlineStr">
         <is>
-          <t>HHI=0.0759  ·  effective N pairs=13.2  ·  max pair=19.05% of gross</t>
+          <t>HHI=0.1132  ·  effective N pairs=8.8  ·  max pair=23.66% of gross</t>
         </is>
       </c>
     </row>
@@ -9979,108 +9979,108 @@
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>KLAC</t>
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>370955.58</v>
+        <v>2114643.6</v>
       </c>
       <c r="C6" s="4" t="n">
-        <v>370955.58</v>
+        <v>2114643.6</v>
       </c>
       <c r="D6" s="23" t="n">
-        <v>36.91</v>
+        <v>210.45</v>
       </c>
       <c r="E6" s="23" t="n">
-        <v>10.16</v>
+        <v>38.08</v>
       </c>
       <c r="F6" s="26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="12" t="inlineStr">
         <is>
-          <t>BWA</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="B7" s="13" t="n">
-        <v>335261.08</v>
+        <v>370955.58</v>
       </c>
       <c r="C7" s="13" t="n">
-        <v>335261.08</v>
+        <v>370955.58</v>
       </c>
       <c r="D7" s="21" t="n">
-        <v>33.36</v>
+        <v>36.92</v>
       </c>
       <c r="E7" s="21" t="n">
-        <v>9.19</v>
+        <v>6.68</v>
       </c>
       <c r="F7" s="28" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
         <is>
-          <t>AWK</t>
+          <t>BWA</t>
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>324143.88</v>
-      </c>
-      <c r="C8" s="19" t="n">
-        <v>-324143.88</v>
+        <v>335261.08</v>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>335261.08</v>
       </c>
       <c r="D8" s="23" t="n">
-        <v>32.26</v>
+        <v>33.37</v>
       </c>
       <c r="E8" s="23" t="n">
-        <v>8.880000000000001</v>
+        <v>6.04</v>
       </c>
       <c r="F8" s="26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>LRCX</t>
+          <t>AWK</t>
         </is>
       </c>
       <c r="B9" s="13" t="n">
-        <v>273357.44</v>
-      </c>
-      <c r="C9" s="13" t="n">
-        <v>273357.44</v>
+        <v>324143.88</v>
+      </c>
+      <c r="C9" s="18" t="n">
+        <v>-324143.88</v>
       </c>
       <c r="D9" s="21" t="n">
-        <v>27.2</v>
+        <v>32.26</v>
       </c>
       <c r="E9" s="21" t="n">
-        <v>7.49</v>
+        <v>5.84</v>
       </c>
       <c r="F9" s="28" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
         <is>
-          <t>STLD</t>
+          <t>LRCX</t>
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>262636.36</v>
+        <v>273357.44</v>
       </c>
       <c r="C10" s="4" t="n">
-        <v>262636.36</v>
+        <v>273357.44</v>
       </c>
       <c r="D10" s="23" t="n">
-        <v>26.14</v>
+        <v>27.2</v>
       </c>
       <c r="E10" s="23" t="n">
-        <v>7.2</v>
+        <v>4.92</v>
       </c>
       <c r="F10" s="26" t="n">
         <v>2</v>
@@ -10089,20 +10089,20 @@
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>CSCO</t>
+          <t>STLD</t>
         </is>
       </c>
       <c r="B11" s="13" t="n">
-        <v>221305.92</v>
+        <v>262636.36</v>
       </c>
       <c r="C11" s="13" t="n">
-        <v>221305.92</v>
+        <v>262636.36</v>
       </c>
       <c r="D11" s="21" t="n">
-        <v>22.02</v>
+        <v>26.14</v>
       </c>
       <c r="E11" s="21" t="n">
-        <v>6.06</v>
+        <v>4.73</v>
       </c>
       <c r="F11" s="28" t="n">
         <v>2</v>
@@ -10111,20 +10111,20 @@
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
         <is>
-          <t>KLAC</t>
+          <t>CSCO</t>
         </is>
       </c>
       <c r="B12" s="4" t="n">
-        <v>211464.36</v>
+        <v>221305.92</v>
       </c>
       <c r="C12" s="4" t="n">
-        <v>211464.36</v>
+        <v>221305.92</v>
       </c>
       <c r="D12" s="23" t="n">
-        <v>21.04</v>
+        <v>22.02</v>
       </c>
       <c r="E12" s="23" t="n">
-        <v>5.79</v>
+        <v>3.99</v>
       </c>
       <c r="F12" s="26" t="n">
         <v>2</v>
@@ -10146,7 +10146,7 @@
         <v>16.77</v>
       </c>
       <c r="E13" s="21" t="n">
-        <v>4.62</v>
+        <v>3.04</v>
       </c>
       <c r="F13" s="28" t="n">
         <v>1</v>
@@ -10168,7 +10168,7 @@
         <v>16.47</v>
       </c>
       <c r="E14" s="23" t="n">
-        <v>4.53</v>
+        <v>2.98</v>
       </c>
       <c r="F14" s="26" t="n">
         <v>2</v>
@@ -10190,7 +10190,7 @@
         <v>13.53</v>
       </c>
       <c r="E15" s="21" t="n">
-        <v>3.72</v>
+        <v>2.45</v>
       </c>
       <c r="F15" s="28" t="n">
         <v>2</v>
@@ -10237,16 +10237,16 @@
         </is>
       </c>
       <c r="B20" s="4" t="n">
-        <v>1004974.13</v>
+        <v>2908153.37</v>
       </c>
       <c r="C20" s="4" t="n">
         <v>134767.54</v>
       </c>
       <c r="D20" s="4" t="n">
-        <v>870206.59</v>
+        <v>2773385.83</v>
       </c>
       <c r="E20" s="7" t="n">
-        <v>23.84</v>
+        <v>49.94</v>
       </c>
     </row>
     <row r="21">
@@ -10265,7 +10265,7 @@
         <v>428116.78</v>
       </c>
       <c r="E21" s="17" t="n">
-        <v>11.73</v>
+        <v>7.71</v>
       </c>
     </row>
     <row r="22">
@@ -10284,7 +10284,7 @@
         <v>-425206.2</v>
       </c>
       <c r="E22" s="7" t="n">
-        <v>-11.65</v>
+        <v>-7.66</v>
       </c>
     </row>
     <row r="23">
@@ -10303,7 +10303,7 @@
         <v>371626.8</v>
       </c>
       <c r="E23" s="17" t="n">
-        <v>10.18</v>
+        <v>6.69</v>
       </c>
     </row>
     <row r="24">
@@ -10322,7 +10322,7 @@
         <v>-324143.88</v>
       </c>
       <c r="E24" s="7" t="n">
-        <v>-8.880000000000001</v>
+        <v>-5.84</v>
       </c>
     </row>
     <row r="25">
@@ -10341,7 +10341,7 @@
         <v>267364.9</v>
       </c>
       <c r="E25" s="17" t="n">
-        <v>7.33</v>
+        <v>4.81</v>
       </c>
     </row>
     <row r="26">
@@ -10360,7 +10360,7 @@
         <v>-186748.67</v>
       </c>
       <c r="E26" s="7" t="n">
-        <v>-5.12</v>
+        <v>-3.36</v>
       </c>
     </row>
   </sheetData>
@@ -10398,7 +10398,7 @@
         </is>
       </c>
       <c r="B3" s="5" t="n">
-        <v>2.664</v>
+        <v>7.123</v>
       </c>
     </row>
     <row r="4">
@@ -10408,7 +10408,7 @@
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>3.718</v>
+        <v>8.177</v>
       </c>
     </row>
     <row r="5">
@@ -10418,7 +10418,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>98.48999999999999</v>
+        <v>287.9</v>
       </c>
     </row>
     <row r="6">
@@ -10459,7 +10459,7 @@
         </is>
       </c>
       <c r="B10" s="23" t="n">
-        <v>23.84</v>
+        <v>49.94</v>
       </c>
     </row>
     <row r="11">
@@ -10469,7 +10469,7 @@
         </is>
       </c>
       <c r="B11" s="21" t="n">
-        <v>11.73</v>
+        <v>7.71</v>
       </c>
     </row>
     <row r="12">
@@ -10479,7 +10479,7 @@
         </is>
       </c>
       <c r="B12" s="24" t="n">
-        <v>-11.65</v>
+        <v>-7.66</v>
       </c>
     </row>
     <row r="13">
@@ -10489,7 +10489,7 @@
         </is>
       </c>
       <c r="B13" s="21" t="n">
-        <v>10.18</v>
+        <v>6.69</v>
       </c>
     </row>
     <row r="14">
@@ -10499,7 +10499,7 @@
         </is>
       </c>
       <c r="B14" s="24" t="n">
-        <v>-8.880000000000001</v>
+        <v>-5.84</v>
       </c>
     </row>
     <row r="15">
@@ -10509,7 +10509,7 @@
         </is>
       </c>
       <c r="B15" s="21" t="n">
-        <v>7.33</v>
+        <v>4.81</v>
       </c>
     </row>
     <row r="16">
@@ -10519,7 +10519,7 @@
         </is>
       </c>
       <c r="B16" s="24" t="n">
-        <v>-5.12</v>
+        <v>-3.36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
RiskManager: retroactive split adjustment for PriceDataStore pre-split prices
When signal_date < split execution_date, PriceDataStore weekly cache
returns pre-split prices (e.g. KLAC $1940 instead of $194). But
adjust_position_view converts positions to post-split (670 shares,
$201 open_price). This mismatch caused $2M phantom unrealized PnL
in risk reports for 6/1-6/5.

Fix: after heal_split_cliff, check if any split-affected ticker has
its entire price series ending before execution_date. If so (and
heal_split_cliff didn't already fix it), divide all prices by the
split factor. Uses _healed_set to avoid double-adjustment.

Result: 6/1 diff improved from $1.9M to +$584 (OK).
11/15 dates now within $2k alignment.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/trading_signals/risk_management/risk_workbook_20260602_153038.xlsx
+++ b/trading_signals/risk_management/risk_workbook_20260602_153038.xlsx
@@ -734,7 +734,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Signal date 2026-06-01  ·  Generated 2026-06-25T01:34:59  ·  Scope: MRPT+MTFS pairs book (model-based, broker-reconciled)</t>
+          <t>Signal date 2026-06-01  ·  Generated 2026-06-25T01:48:24  ·  Scope: MRPT+MTFS pairs book (model-based, broker-reconciled)</t>
         </is>
       </c>
     </row>
@@ -755,7 +755,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>5.526</v>
+        <v>3.632</v>
       </c>
     </row>
     <row r="6">
@@ -764,8 +764,8 @@
           <t>Net leverage (x)</t>
         </is>
       </c>
-      <c r="B6" s="5" t="n">
-        <v>2.89</v>
+      <c r="B6" s="6" t="n">
+        <v>0.996</v>
       </c>
     </row>
     <row r="7">
@@ -775,7 +775,7 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>7.123</v>
+        <v>2.664</v>
       </c>
     </row>
     <row r="8">
@@ -785,7 +785,7 @@
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>117196.95</v>
+        <v>44873.5</v>
       </c>
     </row>
     <row r="9">
@@ -795,7 +795,7 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>11.66</v>
+        <v>4.47</v>
       </c>
     </row>
     <row r="10">
@@ -805,7 +805,7 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>112.56</v>
+        <v>43.1</v>
       </c>
     </row>
     <row r="11">
@@ -857,7 +857,7 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>5.526</v>
+        <v>3.632</v>
       </c>
     </row>
     <row r="16">
@@ -868,7 +868,7 @@
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>KLAC (210.45% NAV)</t>
+          <t>MS (36.92% NAV)</t>
         </is>
       </c>
     </row>
@@ -879,7 +879,7 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>49.94</v>
+        <v>23.84</v>
       </c>
     </row>
     <row r="18">
@@ -899,7 +899,7 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="20">
@@ -950,7 +950,7 @@
         </is>
       </c>
       <c r="B3" s="4" t="n">
-        <v>117196.95</v>
+        <v>44873.5</v>
       </c>
     </row>
     <row r="4">
@@ -960,7 +960,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>165714.35</v>
+        <v>63450.31</v>
       </c>
     </row>
     <row r="5">
@@ -970,7 +970,7 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>1130968.93</v>
+        <v>433036.27</v>
       </c>
     </row>
     <row r="6">
@@ -980,7 +980,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>112.56</v>
+        <v>43.1</v>
       </c>
     </row>
     <row r="7">
@@ -990,7 +990,7 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>95957.89</v>
+        <v>37348.6</v>
       </c>
     </row>
     <row r="8">
@@ -1000,7 +1000,7 @@
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>115645.66</v>
+        <v>43745.98</v>
       </c>
     </row>
     <row r="10">
@@ -1030,131 +1030,131 @@
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
         <is>
-          <t>KLAC/REGN</t>
+          <t>MS/AWK</t>
         </is>
       </c>
       <c r="B12" s="4" t="n">
-        <v>53132.94</v>
+        <v>10307.82</v>
       </c>
       <c r="C12" s="7" t="n">
-        <v>45.34</v>
+        <v>22.97</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="12" t="inlineStr">
         <is>
-          <t>KLAC/LOW</t>
+          <t>LRCX/BSX</t>
         </is>
       </c>
       <c r="B13" s="13" t="n">
-        <v>32641.93</v>
+        <v>5858.42</v>
       </c>
       <c r="C13" s="17" t="n">
-        <v>27.85</v>
+        <v>13.06</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="10" t="inlineStr">
         <is>
-          <t>MS/AWK</t>
+          <t>LRCX/RMD</t>
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>8063.49</v>
+        <v>4589.39</v>
       </c>
       <c r="C14" s="7" t="n">
-        <v>6.88</v>
+        <v>10.23</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
         <is>
-          <t>LRCX/BSX</t>
+          <t>KLAC/REGN</t>
         </is>
       </c>
       <c r="B15" s="13" t="n">
-        <v>5775</v>
+        <v>3838.46</v>
       </c>
       <c r="C15" s="17" t="n">
-        <v>4.93</v>
+        <v>8.550000000000001</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>LRCX/RMD</t>
+          <t>STLD/HII</t>
         </is>
       </c>
       <c r="B16" s="4" t="n">
-        <v>4939.71</v>
+        <v>3067.05</v>
       </c>
       <c r="C16" s="7" t="n">
-        <v>4.21</v>
+        <v>6.83</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="12" t="inlineStr">
         <is>
-          <t>STLD/HII</t>
+          <t>STLD/ISRG</t>
         </is>
       </c>
       <c r="B17" s="13" t="n">
-        <v>2029.07</v>
+        <v>2481.21</v>
       </c>
       <c r="C17" s="17" t="n">
-        <v>1.73</v>
+        <v>5.53</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="10" t="inlineStr">
         <is>
-          <t>STLD/ISRG</t>
+          <t>CI/MTD</t>
         </is>
       </c>
       <c r="B18" s="4" t="n">
-        <v>1776.67</v>
+        <v>1936.6</v>
       </c>
       <c r="C18" s="7" t="n">
-        <v>1.52</v>
+        <v>4.32</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
         <is>
-          <t>ODFL/MKTX</t>
+          <t>NUE/MKTX</t>
         </is>
       </c>
       <c r="B19" s="13" t="n">
-        <v>1547.72</v>
+        <v>1931.05</v>
       </c>
       <c r="C19" s="17" t="n">
-        <v>1.32</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="10" t="inlineStr">
         <is>
-          <t>NUE/MKTX</t>
+          <t>KLAC/LOW</t>
         </is>
       </c>
       <c r="B20" s="4" t="n">
-        <v>1513.96</v>
+        <v>1922.89</v>
       </c>
       <c r="C20" s="7" t="n">
-        <v>1.29</v>
+        <v>4.29</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="12" t="inlineStr">
         <is>
-          <t>NUE/INTU</t>
+          <t>ODFL/MKTX</t>
         </is>
       </c>
       <c r="B21" s="13" t="n">
-        <v>1422.88</v>
+        <v>1813.36</v>
       </c>
       <c r="C21" s="17" t="n">
-        <v>1.21</v>
+        <v>4.04</v>
       </c>
     </row>
     <row r="22">
@@ -1164,62 +1164,62 @@
         </is>
       </c>
       <c r="B22" s="4" t="n">
-        <v>1154.13</v>
+        <v>1652</v>
       </c>
       <c r="C22" s="7" t="n">
-        <v>0.98</v>
+        <v>3.68</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="12" t="inlineStr">
         <is>
-          <t>CI/MTD</t>
+          <t>NUE/INTU</t>
         </is>
       </c>
       <c r="B23" s="13" t="n">
-        <v>1031.91</v>
+        <v>1450.71</v>
       </c>
       <c r="C23" s="17" t="n">
-        <v>0.88</v>
+        <v>3.23</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="10" t="inlineStr">
         <is>
-          <t>BWA/CME</t>
+          <t>FFIV/VLTO</t>
         </is>
       </c>
       <c r="B24" s="4" t="n">
-        <v>896.4299999999999</v>
+        <v>1148.07</v>
       </c>
       <c r="C24" s="7" t="n">
-        <v>0.76</v>
+        <v>2.56</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="12" t="inlineStr">
         <is>
-          <t>FFIV/VLTO</t>
+          <t>BWA/CME</t>
         </is>
       </c>
       <c r="B25" s="13" t="n">
-        <v>769.09</v>
+        <v>1025.02</v>
       </c>
       <c r="C25" s="17" t="n">
-        <v>0.66</v>
+        <v>2.28</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="10" t="inlineStr">
         <is>
-          <t>ODFL/JKHY</t>
+          <t>ORCL/LOW</t>
         </is>
       </c>
       <c r="B26" s="4" t="n">
-        <v>471.02</v>
+        <v>889.2</v>
       </c>
       <c r="C26" s="7" t="n">
-        <v>0.4</v>
+        <v>1.98</v>
       </c>
     </row>
   </sheetData>
@@ -1470,7 +1470,7 @@
         <v>670</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>1010394</v>
+        <v>10103938</v>
       </c>
       <c r="E14" s="7" t="n">
         <v>0</v>
@@ -1554,7 +1554,7 @@
         <v>420</v>
       </c>
       <c r="D18" s="4" t="n">
-        <v>1010394</v>
+        <v>10103938</v>
       </c>
       <c r="E18" s="7" t="n">
         <v>0</v>
@@ -1655,10 +1655,10 @@
         </is>
       </c>
       <c r="B4" s="19" t="n">
-        <v>-357862.16</v>
+        <v>-133840.35</v>
       </c>
       <c r="C4" s="24" t="n">
-        <v>-35.62</v>
+        <v>-13.32</v>
       </c>
     </row>
     <row r="5">
@@ -1668,10 +1668,10 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>-715724.3199999999</v>
+        <v>-267680.69</v>
       </c>
       <c r="C5" s="22" t="n">
-        <v>-71.23</v>
+        <v>-26.64</v>
       </c>
     </row>
     <row r="6">
@@ -1681,10 +1681,10 @@
         </is>
       </c>
       <c r="B6" s="19" t="n">
-        <v>-357862.16</v>
+        <v>-133840.35</v>
       </c>
       <c r="C6" s="24" t="n">
-        <v>-35.62</v>
+        <v>-13.32</v>
       </c>
     </row>
     <row r="7">
@@ -1694,10 +1694,10 @@
         </is>
       </c>
       <c r="B7" s="18" t="n">
-        <v>-277338.58</v>
+        <v>-87020.66</v>
       </c>
       <c r="C7" s="22" t="n">
-        <v>-27.6</v>
+        <v>-8.66</v>
       </c>
     </row>
   </sheetData>
@@ -1828,7 +1828,7 @@
         </is>
       </c>
       <c r="C6" s="34" t="n">
-        <v>12.56</v>
+        <v>8.109999999999999</v>
       </c>
       <c r="D6" s="34" t="n">
         <v>3</v>
@@ -1854,7 +1854,7 @@
         </is>
       </c>
       <c r="C7" s="34" t="n">
-        <v>6.76</v>
+        <v>2.31</v>
       </c>
       <c r="D7" s="34" t="n">
         <v>0.5</v>
@@ -1876,11 +1876,11 @@
       </c>
       <c r="B8" s="34" t="inlineStr">
         <is>
-          <t>KLAC</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="C8" s="34" t="n">
-        <v>210.45</v>
+        <v>36.92</v>
       </c>
       <c r="D8" s="34" t="n">
         <v>15</v>
@@ -1902,11 +1902,11 @@
       </c>
       <c r="B9" s="34" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>BWA</t>
         </is>
       </c>
       <c r="C9" s="34" t="n">
-        <v>36.92</v>
+        <v>33.37</v>
       </c>
       <c r="D9" s="34" t="n">
         <v>15</v>
@@ -1928,11 +1928,11 @@
       </c>
       <c r="B10" s="34" t="inlineStr">
         <is>
-          <t>BWA</t>
+          <t>AWK</t>
         </is>
       </c>
       <c r="C10" s="34" t="n">
-        <v>33.37</v>
+        <v>32.26</v>
       </c>
       <c r="D10" s="34" t="n">
         <v>15</v>
@@ -1947,54 +1947,54 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="35" t="inlineStr">
+      <c r="A11" s="31" t="inlineStr">
         <is>
           <t>sector_net</t>
         </is>
       </c>
-      <c r="B11" s="36" t="inlineStr">
+      <c r="B11" s="32" t="inlineStr">
         <is>
           <t>tech</t>
         </is>
       </c>
-      <c r="C11" s="36" t="n">
-        <v>49.94</v>
-      </c>
-      <c r="D11" s="36" t="n">
+      <c r="C11" s="32" t="n">
+        <v>23.84</v>
+      </c>
+      <c r="D11" s="32" t="n">
         <v>30</v>
       </c>
-      <c r="E11" s="36" t="n">
+      <c r="E11" s="32" t="n">
         <v>50</v>
       </c>
-      <c r="F11" s="36" t="inlineStr">
-        <is>
-          <t>amber</t>
+      <c r="F11" s="32" t="inlineStr">
+        <is>
+          <t>green</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="35" t="inlineStr">
+      <c r="A12" s="31" t="inlineStr">
         <is>
           <t>max_pair</t>
         </is>
       </c>
-      <c r="B12" s="36" t="inlineStr">
+      <c r="B12" s="32" t="inlineStr">
         <is>
           <t>combined</t>
         </is>
       </c>
-      <c r="C12" s="36" t="n">
-        <v>23.66</v>
-      </c>
-      <c r="D12" s="36" t="n">
+      <c r="C12" s="32" t="n">
+        <v>19.05</v>
+      </c>
+      <c r="D12" s="32" t="n">
         <v>20</v>
       </c>
-      <c r="E12" s="36" t="n">
+      <c r="E12" s="32" t="n">
         <v>35</v>
       </c>
-      <c r="F12" s="36" t="inlineStr">
-        <is>
-          <t>amber</t>
+      <c r="F12" s="32" t="inlineStr">
+        <is>
+          <t>green</t>
         </is>
       </c>
     </row>
@@ -2010,7 +2010,7 @@
         </is>
       </c>
       <c r="C13" s="34" t="n">
-        <v>7.12</v>
+        <v>2.66</v>
       </c>
       <c r="D13" s="34" t="n">
         <v>0.3</v>
@@ -2025,28 +2025,28 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="33" t="inlineStr">
+      <c r="A14" s="35" t="inlineStr">
         <is>
           <t>var_95_1d</t>
         </is>
       </c>
-      <c r="B14" s="34" t="inlineStr">
+      <c r="B14" s="36" t="inlineStr">
         <is>
           <t>combined</t>
         </is>
       </c>
-      <c r="C14" s="34" t="n">
-        <v>11.66</v>
-      </c>
-      <c r="D14" s="34" t="n">
+      <c r="C14" s="36" t="n">
+        <v>4.47</v>
+      </c>
+      <c r="D14" s="36" t="n">
         <v>3</v>
       </c>
-      <c r="E14" s="34" t="n">
+      <c r="E14" s="36" t="n">
         <v>5</v>
       </c>
-      <c r="F14" s="34" t="inlineStr">
-        <is>
-          <t>red</t>
+      <c r="F14" s="36" t="inlineStr">
+        <is>
+          <t>amber</t>
         </is>
       </c>
     </row>
@@ -2563,10 +2563,10 @@
         <v>670</v>
       </c>
       <c r="F12" s="13" t="n">
-        <v>1940.04</v>
+        <v>194</v>
       </c>
       <c r="G12" s="13" t="n">
-        <v>1299826.8</v>
+        <v>129982.68</v>
       </c>
       <c r="H12" s="17" t="inlineStr">
         <is>
@@ -2739,10 +2739,10 @@
         <v>420</v>
       </c>
       <c r="F16" s="13" t="n">
-        <v>1940.04</v>
+        <v>194</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>814816.8</v>
+        <v>81481.67999999999</v>
       </c>
       <c r="H16" s="17" t="inlineStr">
         <is>
@@ -4063,11 +4063,11 @@
           <t>KLAC/REGN</t>
         </is>
       </c>
-      <c r="C8" s="13" t="n">
-        <v>1165844.75</v>
+      <c r="C8" s="18" t="n">
+        <v>-3999.37</v>
       </c>
       <c r="D8" s="13" t="n">
-        <v>1313641.98</v>
+        <v>143797.86</v>
       </c>
       <c r="E8" s="17" t="n">
         <v>0</v>
@@ -4126,10 +4126,10 @@
         </is>
       </c>
       <c r="C10" s="13" t="n">
-        <v>737760.38</v>
+        <v>4425.26</v>
       </c>
       <c r="D10" s="13" t="n">
-        <v>894158.2</v>
+        <v>160823.08</v>
       </c>
       <c r="E10" s="17" t="n">
         <v>0</v>
@@ -4801,101 +4801,101 @@
     <row r="13">
       <c r="A13" s="10" t="inlineStr">
         <is>
-          <t>KLAC/REGN</t>
+          <t>MS/AWK</t>
         </is>
       </c>
       <c r="B13" s="7" t="n">
-        <v>45.34</v>
+        <v>22.97</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="12" t="inlineStr">
         <is>
-          <t>KLAC/LOW</t>
+          <t>LRCX/BSX</t>
         </is>
       </c>
       <c r="B14" s="17" t="n">
-        <v>27.85</v>
+        <v>13.06</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="10" t="inlineStr">
         <is>
-          <t>MS/AWK</t>
+          <t>LRCX/RMD</t>
         </is>
       </c>
       <c r="B15" s="7" t="n">
-        <v>6.88</v>
+        <v>10.23</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="12" t="inlineStr">
         <is>
-          <t>LRCX/BSX</t>
+          <t>KLAC/REGN</t>
         </is>
       </c>
       <c r="B16" s="17" t="n">
-        <v>4.93</v>
+        <v>8.550000000000001</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="10" t="inlineStr">
         <is>
-          <t>LRCX/RMD</t>
+          <t>STLD/HII</t>
         </is>
       </c>
       <c r="B17" s="7" t="n">
-        <v>4.21</v>
+        <v>6.83</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="12" t="inlineStr">
         <is>
-          <t>STLD/HII</t>
+          <t>STLD/ISRG</t>
         </is>
       </c>
       <c r="B18" s="17" t="n">
-        <v>1.73</v>
+        <v>5.53</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="10" t="inlineStr">
         <is>
-          <t>STLD/ISRG</t>
+          <t>CI/MTD</t>
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>1.52</v>
+        <v>4.32</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="12" t="inlineStr">
         <is>
-          <t>ODFL/MKTX</t>
+          <t>NUE/MKTX</t>
         </is>
       </c>
       <c r="B20" s="17" t="n">
-        <v>1.32</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="10" t="inlineStr">
         <is>
-          <t>NUE/MKTX</t>
+          <t>KLAC/LOW</t>
         </is>
       </c>
       <c r="B21" s="7" t="n">
-        <v>1.29</v>
+        <v>4.29</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="12" t="inlineStr">
         <is>
-          <t>NUE/INTU</t>
+          <t>ODFL/MKTX</t>
         </is>
       </c>
       <c r="B22" s="17" t="n">
-        <v>1.21</v>
+        <v>4.04</v>
       </c>
     </row>
     <row r="23">
@@ -4905,47 +4905,47 @@
         </is>
       </c>
       <c r="B23" s="7" t="n">
-        <v>0.98</v>
+        <v>3.68</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="12" t="inlineStr">
         <is>
-          <t>CI/MTD</t>
+          <t>NUE/INTU</t>
         </is>
       </c>
       <c r="B24" s="17" t="n">
-        <v>0.88</v>
+        <v>3.23</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="10" t="inlineStr">
         <is>
-          <t>BWA/CME</t>
+          <t>FFIV/VLTO</t>
         </is>
       </c>
       <c r="B25" s="7" t="n">
-        <v>0.76</v>
+        <v>2.56</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="12" t="inlineStr">
         <is>
-          <t>FFIV/VLTO</t>
+          <t>BWA/CME</t>
         </is>
       </c>
       <c r="B26" s="17" t="n">
-        <v>0.66</v>
+        <v>2.28</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="10" t="inlineStr">
         <is>
-          <t>ODFL/JKHY</t>
+          <t>ORCL/LOW</t>
         </is>
       </c>
       <c r="B27" s="7" t="n">
-        <v>0.4</v>
+        <v>1.98</v>
       </c>
     </row>
   </sheetData>
@@ -5441,7 +5441,7 @@
         <v>3.36</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>5.526</v>
+        <v>3.632</v>
       </c>
     </row>
     <row r="10">
@@ -5509,7 +5509,7 @@
         <v>0.37</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>12.559</v>
+        <v>8.108000000000001</v>
       </c>
     </row>
   </sheetData>
@@ -5622,10 +5622,10 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>4228666.25</v>
+        <v>2325487.01</v>
       </c>
       <c r="C7" s="4" t="n">
-        <v>3425427.49</v>
+        <v>1534422.46</v>
       </c>
       <c r="D7" s="4" t="n">
         <v>1877143.41</v>
@@ -5641,10 +5641,10 @@
         </is>
       </c>
       <c r="B8" s="13" t="n">
-        <v>5579422.35</v>
+        <v>3676243.11</v>
       </c>
       <c r="C8" s="13" t="n">
-        <v>4394438.85</v>
+        <v>2503433.82</v>
       </c>
       <c r="D8" s="13" t="n">
         <v>3443683.26</v>
@@ -5679,10 +5679,10 @@
         </is>
       </c>
       <c r="B10" s="13" t="n">
-        <v>3250344.25</v>
+        <v>1347165.01</v>
       </c>
       <c r="C10" s="13" t="n">
-        <v>2455194.43</v>
+        <v>564189.4</v>
       </c>
       <c r="D10" s="13" t="n">
         <v>911068.84</v>
@@ -5698,10 +5698,10 @@
         </is>
       </c>
       <c r="B11" s="4" t="n">
-        <v>4574614.94</v>
+        <v>2671435.7</v>
       </c>
       <c r="C11" s="4" t="n">
-        <v>3405205.57</v>
+        <v>1514200.54</v>
       </c>
       <c r="D11" s="4" t="n">
         <v>2446892.22</v>
@@ -5736,10 +5736,10 @@
         </is>
       </c>
       <c r="B13" s="7" t="n">
-        <v>5.526</v>
+        <v>3.632</v>
       </c>
       <c r="C13" s="7" t="n">
-        <v>4.423</v>
+        <v>2.511</v>
       </c>
       <c r="D13" s="7" t="n">
         <v>3.424</v>
@@ -5755,10 +5755,10 @@
         </is>
       </c>
       <c r="B14" s="17" t="n">
-        <v>2.89</v>
+        <v>0.996</v>
       </c>
       <c r="C14" s="17" t="n">
-        <v>2.502</v>
+        <v>0.591</v>
       </c>
       <c r="D14" s="17" t="n">
         <v>0.342</v>
@@ -5774,10 +5774,10 @@
         </is>
       </c>
       <c r="B15" s="4" t="n">
-        <v>1110587.39</v>
+        <v>729951.54</v>
       </c>
       <c r="C15" s="4" t="n">
-        <v>875087.73</v>
+        <v>496886.72</v>
       </c>
       <c r="D15" s="4" t="n">
         <v>682593.36</v>
@@ -5792,11 +5792,11 @@
           <t>Excess Liquidity 超额流动性</t>
         </is>
       </c>
-      <c r="B16" s="18" t="n">
-        <v>-105779.98</v>
+      <c r="B16" s="13" t="n">
+        <v>274855.87</v>
       </c>
       <c r="C16" s="13" t="n">
-        <v>114145.55</v>
+        <v>492346.56</v>
       </c>
       <c r="D16" s="13" t="n">
         <v>314197.68</v>
@@ -5815,7 +5815,7 @@
         <v>0</v>
       </c>
       <c r="C17" s="7" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="D17" s="7" t="n">
         <v>0</v>
@@ -5903,10 +5903,10 @@
         </is>
       </c>
       <c r="B23" s="4" t="n">
-        <v>4228666.25</v>
+        <v>2325487.01</v>
       </c>
       <c r="C23" s="4" t="n">
-        <v>3425427.49</v>
+        <v>1534422.46</v>
       </c>
       <c r="D23" s="4" t="n">
         <v>1877143.41</v>
@@ -5922,10 +5922,10 @@
         </is>
       </c>
       <c r="B24" s="13" t="n">
-        <v>3223858.84</v>
+        <v>1320679.6</v>
       </c>
       <c r="C24" s="13" t="n">
-        <v>2436194.21</v>
+        <v>545189.1800000001</v>
       </c>
       <c r="D24" s="13" t="n">
         <v>880352.37</v>
@@ -6784,10 +6784,10 @@
         </is>
       </c>
       <c r="B75" s="4" t="n">
-        <v>4131613.51</v>
+        <v>2228434.27</v>
       </c>
       <c r="C75" s="4" t="n">
-        <v>3273399.55</v>
+        <v>1382394.52</v>
       </c>
       <c r="D75" s="4" t="n">
         <v>1559846.18</v>
@@ -6803,10 +6803,10 @@
         </is>
       </c>
       <c r="B76" s="13" t="n">
-        <v>5395111.39</v>
+        <v>3491932.15</v>
       </c>
       <c r="C76" s="13" t="n">
-        <v>4090701.74</v>
+        <v>2199696.71</v>
       </c>
       <c r="D76" s="13" t="n">
         <v>2713130.28</v>
@@ -6841,10 +6841,10 @@
         </is>
       </c>
       <c r="B78" s="13" t="n">
-        <v>3728791</v>
+        <v>1825611.76</v>
       </c>
       <c r="C78" s="13" t="n">
-        <v>2874457.97</v>
+        <v>983452.9399999999</v>
       </c>
       <c r="D78" s="13" t="n">
         <v>1159739.14</v>
@@ -6860,10 +6860,10 @@
         </is>
       </c>
       <c r="B79" s="4" t="n">
-        <v>4967514.41</v>
+        <v>3064335.17</v>
       </c>
       <c r="C79" s="4" t="n">
-        <v>3675734.63</v>
+        <v>1784729.6</v>
       </c>
       <c r="D79" s="4" t="n">
         <v>2290409.83</v>
@@ -6898,10 +6898,10 @@
         </is>
       </c>
       <c r="B81" s="7" t="n">
-        <v>12.559</v>
+        <v>8.108000000000001</v>
       </c>
       <c r="C81" s="7" t="n">
-        <v>9.819000000000001</v>
+        <v>5.262</v>
       </c>
       <c r="D81" s="7" t="n">
         <v>6.365</v>
@@ -6917,10 +6917,10 @@
         </is>
       </c>
       <c r="B82" s="17" t="n">
-        <v>6.765</v>
+        <v>2.315</v>
       </c>
       <c r="C82" s="17" t="n">
-        <v>5.957</v>
+        <v>1.4</v>
       </c>
       <c r="D82" s="17" t="n">
         <v>1.015</v>
@@ -6936,10 +6936,10 @@
         </is>
       </c>
       <c r="B83" s="4" t="n">
-        <v>1074067.38</v>
+        <v>693431.54</v>
       </c>
       <c r="C83" s="4" t="n">
-        <v>814935.24</v>
+        <v>436734.24</v>
       </c>
       <c r="D83" s="4" t="n">
         <v>538103.37</v>
@@ -6955,10 +6955,10 @@
         </is>
       </c>
       <c r="B84" s="18" t="n">
-        <v>-646470.4</v>
+        <v>-265834.56</v>
       </c>
       <c r="C84" s="18" t="n">
-        <v>-399968.13</v>
+        <v>-21767.13</v>
       </c>
       <c r="D84" s="18" t="n">
         <v>-115382.92</v>
@@ -6974,7 +6974,7 @@
         </is>
       </c>
       <c r="B85" s="7" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="C85" s="7" t="n">
         <v>0</v>
@@ -7065,10 +7065,10 @@
         </is>
       </c>
       <c r="B91" s="4" t="n">
-        <v>4131613.51</v>
+        <v>2228434.27</v>
       </c>
       <c r="C91" s="4" t="n">
-        <v>3273399.55</v>
+        <v>1382394.52</v>
       </c>
       <c r="D91" s="4" t="n">
         <v>1559846.18</v>
@@ -7084,10 +7084,10 @@
         </is>
       </c>
       <c r="B92" s="13" t="n">
-        <v>3704016.53</v>
+        <v>1800837.29</v>
       </c>
       <c r="C92" s="13" t="n">
-        <v>2858432.44</v>
+        <v>967427.41</v>
       </c>
       <c r="D92" s="13" t="n">
         <v>1137125.73</v>
@@ -7377,16 +7377,16 @@
         </is>
       </c>
       <c r="B6" s="13" t="n">
-        <v>445.25</v>
+        <v>184.54</v>
       </c>
       <c r="C6" s="13" t="n">
-        <v>2226.26</v>
+        <v>922.72</v>
       </c>
       <c r="D6" s="13" t="n">
-        <v>9350.309999999999</v>
+        <v>3875.41</v>
       </c>
       <c r="E6" s="13" t="n">
-        <v>64561.63</v>
+        <v>26758.76</v>
       </c>
     </row>
     <row r="7">
@@ -7396,7 +7396,7 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>2001163.55</v>
+        <v>97984.31</v>
       </c>
     </row>
     <row r="9">
@@ -7541,16 +7541,16 @@
         </is>
       </c>
       <c r="B18" s="13" t="n">
-        <v>510.79</v>
+        <v>250.08</v>
       </c>
       <c r="C18" s="13" t="n">
-        <v>2553.97</v>
+        <v>1250.42</v>
       </c>
       <c r="D18" s="13" t="n">
-        <v>10726.66</v>
+        <v>5251.76</v>
       </c>
       <c r="E18" s="13" t="n">
-        <v>74065.03</v>
+        <v>36262.15</v>
       </c>
     </row>
     <row r="19">
@@ -7560,7 +7560,7 @@
         </is>
       </c>
       <c r="B19" s="4" t="n">
-        <v>1987907.71</v>
+        <v>84728.47</v>
       </c>
     </row>
     <row r="21">
@@ -8159,7 +8159,7 @@
         </is>
       </c>
       <c r="B5" s="19" t="n">
-        <v>-2563075.53</v>
+        <v>-659896.29</v>
       </c>
     </row>
     <row r="6">
@@ -8169,7 +8169,7 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>2339275.41</v>
+        <v>436096.17</v>
       </c>
     </row>
     <row r="7">
@@ -9804,28 +9804,28 @@
         <v>1004807.41</v>
       </c>
       <c r="C4" s="4" t="n">
-        <v>4228666.25</v>
+        <v>2325487.01</v>
       </c>
       <c r="D4" s="4" t="n">
         <v>1324270.69</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>5552936.94</v>
+        <v>3649757.7</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>2904395.56</v>
+        <v>1001216.32</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>5.526</v>
+        <v>3.632</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>2.89</v>
+        <v>0.996</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>552.64</v>
+        <v>363.23</v>
       </c>
       <c r="J4" s="5" t="n">
-        <v>276.32</v>
+        <v>181.61</v>
       </c>
       <c r="K4" s="26" t="n">
         <v>19</v>
@@ -9878,28 +9878,28 @@
         <v>427596.98</v>
       </c>
       <c r="C6" s="4" t="n">
-        <v>4131613.51</v>
+        <v>2228434.27</v>
       </c>
       <c r="D6" s="4" t="n">
         <v>1238723.41</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>5370336.92</v>
+        <v>3467157.68</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>2892890.1</v>
+        <v>989710.86</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>12.559</v>
+        <v>8.108000000000001</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>6.765</v>
+        <v>2.315</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>1255.93</v>
+        <v>810.85</v>
       </c>
       <c r="J6" s="5" t="n">
-        <v>627.97</v>
+        <v>405.42</v>
       </c>
       <c r="K6" s="26" t="n">
         <v>18</v>
@@ -9940,7 +9940,7 @@
     <row r="3">
       <c r="A3" s="29" t="inlineStr">
         <is>
-          <t>HHI=0.1132  ·  effective N pairs=8.8  ·  max pair=23.66% of gross</t>
+          <t>HHI=0.0759  ·  effective N pairs=13.2  ·  max pair=19.05% of gross</t>
         </is>
       </c>
     </row>
@@ -9979,108 +9979,108 @@
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
         <is>
-          <t>KLAC</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>2114643.6</v>
+        <v>370955.58</v>
       </c>
       <c r="C6" s="4" t="n">
-        <v>2114643.6</v>
+        <v>370955.58</v>
       </c>
       <c r="D6" s="23" t="n">
-        <v>210.45</v>
+        <v>36.92</v>
       </c>
       <c r="E6" s="23" t="n">
-        <v>38.08</v>
+        <v>10.16</v>
       </c>
       <c r="F6" s="26" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="12" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>BWA</t>
         </is>
       </c>
       <c r="B7" s="13" t="n">
-        <v>370955.58</v>
+        <v>335261.08</v>
       </c>
       <c r="C7" s="13" t="n">
-        <v>370955.58</v>
+        <v>335261.08</v>
       </c>
       <c r="D7" s="21" t="n">
-        <v>36.92</v>
+        <v>33.37</v>
       </c>
       <c r="E7" s="21" t="n">
-        <v>6.68</v>
+        <v>9.19</v>
       </c>
       <c r="F7" s="28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
         <is>
-          <t>BWA</t>
+          <t>AWK</t>
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>335261.08</v>
-      </c>
-      <c r="C8" s="4" t="n">
-        <v>335261.08</v>
+        <v>324143.88</v>
+      </c>
+      <c r="C8" s="19" t="n">
+        <v>-324143.88</v>
       </c>
       <c r="D8" s="23" t="n">
-        <v>33.37</v>
+        <v>32.26</v>
       </c>
       <c r="E8" s="23" t="n">
-        <v>6.04</v>
+        <v>8.880000000000001</v>
       </c>
       <c r="F8" s="26" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>AWK</t>
+          <t>LRCX</t>
         </is>
       </c>
       <c r="B9" s="13" t="n">
-        <v>324143.88</v>
-      </c>
-      <c r="C9" s="18" t="n">
-        <v>-324143.88</v>
+        <v>273357.44</v>
+      </c>
+      <c r="C9" s="13" t="n">
+        <v>273357.44</v>
       </c>
       <c r="D9" s="21" t="n">
-        <v>32.26</v>
+        <v>27.2</v>
       </c>
       <c r="E9" s="21" t="n">
-        <v>5.84</v>
+        <v>7.49</v>
       </c>
       <c r="F9" s="28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
         <is>
-          <t>LRCX</t>
+          <t>STLD</t>
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>273357.44</v>
+        <v>262636.36</v>
       </c>
       <c r="C10" s="4" t="n">
-        <v>273357.44</v>
+        <v>262636.36</v>
       </c>
       <c r="D10" s="23" t="n">
-        <v>27.2</v>
+        <v>26.14</v>
       </c>
       <c r="E10" s="23" t="n">
-        <v>4.92</v>
+        <v>7.2</v>
       </c>
       <c r="F10" s="26" t="n">
         <v>2</v>
@@ -10089,20 +10089,20 @@
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>STLD</t>
+          <t>CSCO</t>
         </is>
       </c>
       <c r="B11" s="13" t="n">
-        <v>262636.36</v>
+        <v>221305.92</v>
       </c>
       <c r="C11" s="13" t="n">
-        <v>262636.36</v>
+        <v>221305.92</v>
       </c>
       <c r="D11" s="21" t="n">
-        <v>26.14</v>
+        <v>22.02</v>
       </c>
       <c r="E11" s="21" t="n">
-        <v>4.73</v>
+        <v>6.06</v>
       </c>
       <c r="F11" s="28" t="n">
         <v>2</v>
@@ -10111,20 +10111,20 @@
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
         <is>
-          <t>CSCO</t>
+          <t>KLAC</t>
         </is>
       </c>
       <c r="B12" s="4" t="n">
-        <v>221305.92</v>
+        <v>211464.36</v>
       </c>
       <c r="C12" s="4" t="n">
-        <v>221305.92</v>
+        <v>211464.36</v>
       </c>
       <c r="D12" s="23" t="n">
-        <v>22.02</v>
+        <v>21.05</v>
       </c>
       <c r="E12" s="23" t="n">
-        <v>3.99</v>
+        <v>5.79</v>
       </c>
       <c r="F12" s="26" t="n">
         <v>2</v>
@@ -10146,7 +10146,7 @@
         <v>16.77</v>
       </c>
       <c r="E13" s="21" t="n">
-        <v>3.04</v>
+        <v>4.62</v>
       </c>
       <c r="F13" s="28" t="n">
         <v>1</v>
@@ -10168,7 +10168,7 @@
         <v>16.47</v>
       </c>
       <c r="E14" s="23" t="n">
-        <v>2.98</v>
+        <v>4.53</v>
       </c>
       <c r="F14" s="26" t="n">
         <v>2</v>
@@ -10190,7 +10190,7 @@
         <v>13.53</v>
       </c>
       <c r="E15" s="21" t="n">
-        <v>2.45</v>
+        <v>3.72</v>
       </c>
       <c r="F15" s="28" t="n">
         <v>2</v>
@@ -10237,16 +10237,16 @@
         </is>
       </c>
       <c r="B20" s="4" t="n">
-        <v>2908153.37</v>
+        <v>1004974.13</v>
       </c>
       <c r="C20" s="4" t="n">
         <v>134767.54</v>
       </c>
       <c r="D20" s="4" t="n">
-        <v>2773385.83</v>
+        <v>870206.59</v>
       </c>
       <c r="E20" s="7" t="n">
-        <v>49.94</v>
+        <v>23.84</v>
       </c>
     </row>
     <row r="21">
@@ -10265,7 +10265,7 @@
         <v>428116.78</v>
       </c>
       <c r="E21" s="17" t="n">
-        <v>7.71</v>
+        <v>11.73</v>
       </c>
     </row>
     <row r="22">
@@ -10284,7 +10284,7 @@
         <v>-425206.2</v>
       </c>
       <c r="E22" s="7" t="n">
-        <v>-7.66</v>
+        <v>-11.65</v>
       </c>
     </row>
     <row r="23">
@@ -10303,7 +10303,7 @@
         <v>371626.8</v>
       </c>
       <c r="E23" s="17" t="n">
-        <v>6.69</v>
+        <v>10.18</v>
       </c>
     </row>
     <row r="24">
@@ -10322,7 +10322,7 @@
         <v>-324143.88</v>
       </c>
       <c r="E24" s="7" t="n">
-        <v>-5.84</v>
+        <v>-8.880000000000001</v>
       </c>
     </row>
     <row r="25">
@@ -10341,7 +10341,7 @@
         <v>267364.9</v>
       </c>
       <c r="E25" s="17" t="n">
-        <v>4.81</v>
+        <v>7.33</v>
       </c>
     </row>
     <row r="26">
@@ -10360,7 +10360,7 @@
         <v>-186748.67</v>
       </c>
       <c r="E26" s="7" t="n">
-        <v>-3.36</v>
+        <v>-5.12</v>
       </c>
     </row>
   </sheetData>
@@ -10398,7 +10398,7 @@
         </is>
       </c>
       <c r="B3" s="5" t="n">
-        <v>7.123</v>
+        <v>2.664</v>
       </c>
     </row>
     <row r="4">
@@ -10408,7 +10408,7 @@
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>8.177</v>
+        <v>3.719</v>
       </c>
     </row>
     <row r="5">
@@ -10418,7 +10418,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>287.9</v>
+        <v>98.5</v>
       </c>
     </row>
     <row r="6">
@@ -10459,7 +10459,7 @@
         </is>
       </c>
       <c r="B10" s="23" t="n">
-        <v>49.94</v>
+        <v>23.84</v>
       </c>
     </row>
     <row r="11">
@@ -10469,7 +10469,7 @@
         </is>
       </c>
       <c r="B11" s="21" t="n">
-        <v>7.71</v>
+        <v>11.73</v>
       </c>
     </row>
     <row r="12">
@@ -10479,7 +10479,7 @@
         </is>
       </c>
       <c r="B12" s="24" t="n">
-        <v>-7.66</v>
+        <v>-11.65</v>
       </c>
     </row>
     <row r="13">
@@ -10489,7 +10489,7 @@
         </is>
       </c>
       <c r="B13" s="21" t="n">
-        <v>6.69</v>
+        <v>10.18</v>
       </c>
     </row>
     <row r="14">
@@ -10499,7 +10499,7 @@
         </is>
       </c>
       <c r="B14" s="24" t="n">
-        <v>-5.84</v>
+        <v>-8.880000000000001</v>
       </c>
     </row>
     <row r="15">
@@ -10509,7 +10509,7 @@
         </is>
       </c>
       <c r="B15" s="21" t="n">
-        <v>4.81</v>
+        <v>7.33</v>
       </c>
     </row>
     <row r="16">
@@ -10519,7 +10519,7 @@
         </is>
       </c>
       <c r="B16" s="24" t="n">
-        <v>-3.36</v>
+        <v>-5.12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>